<commit_message>
add net and update goog
</commit_message>
<xml_diff>
--- a/GOOG.xlsx
+++ b/GOOG.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shkre\code\models\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffe\Documents\GitHub\martinshkreli-models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6EA2A4-4AF5-4CB8-9C17-F3FC30D17748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{485A8EDC-61BB-4A49-93FD-33DCA087ECD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23250" yWindow="45" windowWidth="28395" windowHeight="20910" activeTab="1" xr2:uid="{605BC9F4-5436-4082-9BF9-F0067EF1EC53}"/>
+    <workbookView xWindow="16140" yWindow="90" windowWidth="24285" windowHeight="20805" activeTab="1" xr2:uid="{605BC9F4-5436-4082-9BF9-F0067EF1EC53}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -375,7 +375,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -404,12 +404,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -432,7 +426,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -466,9 +460,6 @@
     </xf>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -601,9 +592,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -641,7 +632,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -747,7 +738,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -889,7 +880,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1216,7 +1207,9 @@
       <c r="S3" s="11"/>
       <c r="T3" s="11"/>
       <c r="U3" s="11"/>
-      <c r="V3" s="11"/>
+      <c r="V3" s="11">
+        <v>150</v>
+      </c>
       <c r="AE3" s="3">
         <v>-169</v>
       </c>
@@ -1235,7 +1228,7 @@
         <v>149</v>
       </c>
       <c r="AJ3" s="3">
-        <f t="shared" ref="AJ3:AJ9" si="3">SUM(O3:R3)</f>
+        <f t="shared" ref="AJ3:AK9" si="3">SUM(O3:R3)</f>
         <v>1960</v>
       </c>
     </row>
@@ -1298,8 +1291,7 @@
         <v>209</v>
       </c>
       <c r="V4" s="11">
-        <f t="shared" si="4"/>
-        <v>226</v>
+        <v>657</v>
       </c>
       <c r="AE4" s="3">
         <v>477</v>
@@ -1323,36 +1315,36 @@
         <v>1068</v>
       </c>
       <c r="AK4" s="3">
-        <f>+AJ4*1.01</f>
-        <v>1078.68</v>
+        <f>SUM(S4:V4)</f>
+        <v>1499</v>
       </c>
       <c r="AL4" s="3">
         <f t="shared" ref="AL4:AR4" si="5">+AK4*1.01</f>
-        <v>1089.4668000000001</v>
+        <v>1513.99</v>
       </c>
       <c r="AM4" s="3">
         <f t="shared" si="5"/>
-        <v>1100.3614680000001</v>
+        <v>1529.1299000000001</v>
       </c>
       <c r="AN4" s="3">
         <f t="shared" si="5"/>
-        <v>1111.3650826800001</v>
+        <v>1544.4211990000001</v>
       </c>
       <c r="AO4" s="3">
         <f t="shared" si="5"/>
-        <v>1122.4787335068002</v>
+        <v>1559.8654109900001</v>
       </c>
       <c r="AP4" s="3">
         <f t="shared" si="5"/>
-        <v>1133.7035208418681</v>
+        <v>1575.4640650999002</v>
       </c>
       <c r="AQ4" s="3">
         <f t="shared" si="5"/>
-        <v>1145.0405560502868</v>
+        <v>1591.2187057508991</v>
       </c>
       <c r="AR4" s="3">
         <f t="shared" si="5"/>
-        <v>1156.4909616107898</v>
+        <v>1607.1308928084081</v>
       </c>
     </row>
     <row r="5" spans="1:44" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -1414,8 +1406,7 @@
         <v>9615.1999999999989</v>
       </c>
       <c r="V5" s="11">
-        <f t="shared" si="6"/>
-        <v>10241</v>
+        <v>9192</v>
       </c>
       <c r="AE5" s="3">
         <v>4056</v>
@@ -1439,36 +1430,36 @@
         <v>26280</v>
       </c>
       <c r="AK5" s="3">
-        <f>+AJ5*1.4</f>
-        <v>36792</v>
+        <f>SUM(S5:V5)</f>
+        <v>35743</v>
       </c>
       <c r="AL5" s="3">
         <f t="shared" ref="AL5" si="7">+AK5*1.4</f>
-        <v>51508.799999999996</v>
+        <v>50040.2</v>
       </c>
       <c r="AM5" s="3">
         <f>+AL5*1.3</f>
-        <v>66961.440000000002</v>
+        <v>65052.26</v>
       </c>
       <c r="AN5" s="3">
         <f>+AM5*1.3</f>
-        <v>87049.872000000003</v>
+        <v>84567.938000000009</v>
       </c>
       <c r="AO5" s="3">
         <f>+AN5*1.3</f>
-        <v>113164.83360000001</v>
+        <v>109938.31940000002</v>
       </c>
       <c r="AP5" s="3">
         <f>+AO5*1.2</f>
-        <v>135797.80032000001</v>
+        <v>131925.98328000001</v>
       </c>
       <c r="AQ5" s="3">
         <f>+AP5*1.2</f>
-        <v>162957.360384</v>
+        <v>158311.179936</v>
       </c>
       <c r="AR5" s="3">
         <f>+AQ5*1.2</f>
-        <v>195548.83246079998</v>
+        <v>189973.41592319999</v>
       </c>
     </row>
     <row r="6" spans="1:44" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -1555,7 +1546,7 @@
         <v>29055</v>
       </c>
       <c r="AK6" s="3">
-        <f>+AJ6*1.03</f>
+        <f>SUM(S6:V6)</f>
         <v>29926.65</v>
       </c>
       <c r="AL6" s="3">
@@ -1646,8 +1637,7 @@
         <v>8659.2000000000007</v>
       </c>
       <c r="V7" s="11">
-        <f>+R7*1.1</f>
-        <v>9322.5</v>
+        <v>8297</v>
       </c>
       <c r="AE7" s="3">
         <v>17616</v>
@@ -1671,36 +1661,36 @@
         <v>32780</v>
       </c>
       <c r="AK7" s="3">
-        <f>+AJ7*1.03</f>
-        <v>33763.4</v>
+        <f>SUM(S7:V7)</f>
+        <v>35032.5</v>
       </c>
       <c r="AL7" s="3">
         <f t="shared" ref="AL7:AR7" si="9">+AK7*1.03</f>
-        <v>34776.302000000003</v>
+        <v>36083.474999999999</v>
       </c>
       <c r="AM7" s="3">
         <f t="shared" si="9"/>
-        <v>35819.591060000006</v>
+        <v>37165.979249999997</v>
       </c>
       <c r="AN7" s="3">
         <f t="shared" si="9"/>
-        <v>36894.178791800005</v>
+        <v>38280.958627499997</v>
       </c>
       <c r="AO7" s="3">
         <f t="shared" si="9"/>
-        <v>38001.004155554008</v>
+        <v>39429.387386324997</v>
       </c>
       <c r="AP7" s="3">
         <f t="shared" si="9"/>
-        <v>39141.034280220629</v>
+        <v>40612.269007914751</v>
       </c>
       <c r="AQ7" s="3">
         <f t="shared" si="9"/>
-        <v>40315.265308627248</v>
+        <v>41830.637078152191</v>
       </c>
       <c r="AR7" s="3">
         <f t="shared" si="9"/>
-        <v>41524.723267886067</v>
+        <v>43085.556190496754</v>
       </c>
     </row>
     <row r="8" spans="1:44" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -1762,8 +1752,7 @@
         <v>7495.26</v>
       </c>
       <c r="V8" s="11">
-        <f>+R8*1.06</f>
-        <v>8440.7800000000007</v>
+        <v>9200</v>
       </c>
       <c r="AE8" s="3">
         <v>8150</v>
@@ -1787,36 +1776,36 @@
         <v>29243</v>
       </c>
       <c r="AK8" s="3">
-        <f>+AJ8*1.05</f>
-        <v>30705.15</v>
+        <f>SUM(S8:V8)</f>
+        <v>31756.800000000003</v>
       </c>
       <c r="AL8" s="3">
         <f t="shared" ref="AL8:AR8" si="10">+AK8*1.05</f>
-        <v>32240.407500000001</v>
+        <v>33344.640000000007</v>
       </c>
       <c r="AM8" s="3">
         <f t="shared" si="10"/>
-        <v>33852.427875000001</v>
+        <v>35011.87200000001</v>
       </c>
       <c r="AN8" s="3">
         <f t="shared" si="10"/>
-        <v>35545.049268750001</v>
+        <v>36762.46560000001</v>
       </c>
       <c r="AO8" s="3">
         <f t="shared" si="10"/>
-        <v>37322.301732187501</v>
+        <v>38600.58888000001</v>
       </c>
       <c r="AP8" s="3">
         <f t="shared" si="10"/>
-        <v>39188.416818796875</v>
+        <v>40530.61832400001</v>
       </c>
       <c r="AQ8" s="3">
         <f t="shared" si="10"/>
-        <v>41147.837659736724</v>
+        <v>42557.149240200015</v>
       </c>
       <c r="AR8" s="3">
         <f t="shared" si="10"/>
-        <v>43205.229542723566</v>
+        <v>44685.006702210019</v>
       </c>
     </row>
     <row r="9" spans="1:44" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -1878,8 +1867,7 @@
         <v>43492.9</v>
       </c>
       <c r="V9" s="11">
-        <f>+R9*1.1</f>
-        <v>46864.4</v>
+        <v>48020</v>
       </c>
       <c r="AE9" s="3">
         <v>69811</v>
@@ -1903,36 +1891,36 @@
         <v>162450</v>
       </c>
       <c r="AK9" s="3">
-        <f>+AJ9*1.1</f>
-        <v>178695</v>
+        <f>SUM(S9:V9)</f>
+        <v>179850.6</v>
       </c>
       <c r="AL9" s="3">
         <f t="shared" ref="AL9:AR9" si="11">+AK9*1.1</f>
-        <v>196564.50000000003</v>
+        <v>197835.66000000003</v>
       </c>
       <c r="AM9" s="3">
         <f t="shared" si="11"/>
-        <v>216220.95000000004</v>
+        <v>217619.22600000005</v>
       </c>
       <c r="AN9" s="3">
         <f t="shared" si="11"/>
-        <v>237843.04500000007</v>
+        <v>239381.14860000007</v>
       </c>
       <c r="AO9" s="3">
         <f t="shared" si="11"/>
-        <v>261627.3495000001</v>
+        <v>263319.2634600001</v>
       </c>
       <c r="AP9" s="3">
         <f t="shared" si="11"/>
-        <v>287790.08445000014</v>
+        <v>289651.18980600015</v>
       </c>
       <c r="AQ9" s="3">
         <f t="shared" si="11"/>
-        <v>316569.09289500018</v>
+        <v>318616.30878660019</v>
       </c>
       <c r="AR9" s="3">
         <f t="shared" si="11"/>
-        <v>348226.00218450022</v>
+        <v>350477.93966526026</v>
       </c>
     </row>
     <row r="10" spans="1:44" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -2015,8 +2003,7 @@
         <v>66749.210000000006</v>
       </c>
       <c r="V10" s="11">
-        <f>SUM(V6:V9)</f>
-        <v>73687.56</v>
+        <v>76311</v>
       </c>
       <c r="AE10" s="11">
         <f t="shared" ref="AE10:AH10" si="16">SUM(AE6:AE9)</f>
@@ -2044,35 +2031,35 @@
       </c>
       <c r="AK10" s="11">
         <f>SUM(AK6:AK9)</f>
-        <v>273090.2</v>
+        <v>276566.55000000005</v>
       </c>
       <c r="AL10" s="11">
         <f t="shared" ref="AL10:AR10" si="17">SUM(AL6:AL9)</f>
-        <v>294405.65900000004</v>
+        <v>298088.22450000001</v>
       </c>
       <c r="AM10" s="11">
         <f t="shared" si="17"/>
-        <v>317642.15192000009</v>
+        <v>321546.26023500005</v>
       </c>
       <c r="AN10" s="11">
         <f t="shared" si="17"/>
-        <v>342983.9315351001</v>
+        <v>347126.23130205006</v>
       </c>
       <c r="AO10" s="11">
         <f t="shared" si="17"/>
-        <v>370633.36361652811</v>
+        <v>375031.94795511162</v>
       </c>
       <c r="AP10" s="11">
         <f t="shared" si="17"/>
-        <v>400812.72502466774</v>
+        <v>405487.26661356504</v>
       </c>
       <c r="AQ10" s="11">
         <f t="shared" si="17"/>
-        <v>433766.18102328375</v>
+        <v>438738.080264872</v>
       </c>
       <c r="AR10" s="11">
         <f t="shared" si="17"/>
-        <v>469761.95970982703</v>
+        <v>475054.50727268425</v>
       </c>
     </row>
     <row r="11" spans="1:44" s="9" customFormat="1" x14ac:dyDescent="0.2">
@@ -2156,7 +2143,7 @@
       </c>
       <c r="V11" s="10">
         <f t="shared" si="21"/>
-        <v>84154.559999999998</v>
+        <v>86310</v>
       </c>
       <c r="W11" s="10"/>
       <c r="X11" s="10"/>
@@ -2202,35 +2189,35 @@
       </c>
       <c r="AK11" s="10">
         <f t="shared" ref="AK11" si="23">AK10+AK5+AK4+AK3</f>
-        <v>310960.88</v>
+        <v>313808.55000000005</v>
       </c>
       <c r="AL11" s="10">
         <f t="shared" ref="AL11" si="24">AL10+AL5+AL4+AL3</f>
-        <v>347003.92580000003</v>
+        <v>349642.41450000001</v>
       </c>
       <c r="AM11" s="10">
         <f t="shared" ref="AM11" si="25">AM10+AM5+AM4+AM3</f>
-        <v>385703.95338800008</v>
+        <v>388127.65013500006</v>
       </c>
       <c r="AN11" s="10">
         <f t="shared" ref="AN11" si="26">AN10+AN5+AN4+AN3</f>
-        <v>431145.16861778009</v>
+        <v>433238.59050105006</v>
       </c>
       <c r="AO11" s="10">
         <f t="shared" ref="AO11" si="27">AO10+AO5+AO4+AO3</f>
-        <v>484920.67595003493</v>
+        <v>486530.13276610168</v>
       </c>
       <c r="AP11" s="10">
         <f t="shared" ref="AP11" si="28">AP10+AP5+AP4+AP3</f>
-        <v>537744.22886550962</v>
+        <v>538988.71395866503</v>
       </c>
       <c r="AQ11" s="10">
         <f t="shared" ref="AQ11" si="29">AQ10+AQ5+AQ4+AQ3</f>
-        <v>597868.581963334</v>
+        <v>598640.47890662285</v>
       </c>
       <c r="AR11" s="10">
         <f t="shared" ref="AR11" si="30">AR10+AR5+AR4+AR3</f>
-        <v>666467.28313223785</v>
+        <v>666635.05408869265</v>
       </c>
     </row>
     <row r="12" spans="1:44" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -2313,35 +2300,35 @@
       </c>
       <c r="AK12" s="3">
         <f>+AK11-AK14</f>
-        <v>136822.78719999999</v>
+        <v>138075.76200000002</v>
       </c>
       <c r="AL12" s="3">
         <f t="shared" ref="AL12:AR12" si="31">+AL11-AL14</f>
-        <v>152681.72735199999</v>
+        <v>153842.66237999999</v>
       </c>
       <c r="AM12" s="3">
         <f t="shared" si="31"/>
-        <v>169709.73949072001</v>
+        <v>170776.16605940001</v>
       </c>
       <c r="AN12" s="3">
         <f t="shared" si="31"/>
-        <v>189703.87419182321</v>
+        <v>190624.979820462</v>
       </c>
       <c r="AO12" s="3">
         <f t="shared" si="31"/>
-        <v>213365.09741801536</v>
+        <v>214073.2584170847</v>
       </c>
       <c r="AP12" s="3">
         <f t="shared" si="31"/>
-        <v>236607.46070082422</v>
+        <v>237155.03414181259</v>
       </c>
       <c r="AQ12" s="3">
         <f t="shared" si="31"/>
-        <v>263062.17606386694</v>
+        <v>263401.81071891403</v>
       </c>
       <c r="AR12" s="3">
         <f t="shared" si="31"/>
-        <v>293245.6045781846</v>
+        <v>293319.42379902472</v>
       </c>
     </row>
     <row r="13" spans="1:44" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -2443,27 +2430,27 @@
       <c r="U14" s="11"/>
       <c r="V14" s="11"/>
       <c r="AB14" s="3">
-        <f>+AB11-AB12</f>
+        <f t="shared" ref="AB14:AG14" si="36">+AB11-AB12</f>
         <v>40310</v>
       </c>
       <c r="AC14" s="3">
-        <f>+AC11-AC12</f>
+        <f t="shared" si="36"/>
         <v>46825</v>
       </c>
       <c r="AD14" s="3">
-        <f>+AD11-AD12</f>
+        <f t="shared" si="36"/>
         <v>55134</v>
       </c>
       <c r="AE14" s="3">
-        <f>+AE11-AE12</f>
+        <f t="shared" si="36"/>
         <v>65272</v>
       </c>
       <c r="AF14" s="3">
-        <f>+AF11-AF12</f>
+        <f t="shared" si="36"/>
         <v>77270</v>
       </c>
       <c r="AG14" s="3">
-        <f>+AG11-AG12</f>
+        <f t="shared" si="36"/>
         <v>89961</v>
       </c>
       <c r="AH14" s="3">
@@ -2471,7 +2458,7 @@
         <v>97795</v>
       </c>
       <c r="AI14" s="3">
-        <f t="shared" ref="AI14" si="36">AI11-AI12</f>
+        <f t="shared" ref="AI14" si="37">AI11-AI12</f>
         <v>146698</v>
       </c>
       <c r="AJ14" s="3">
@@ -2480,35 +2467,35 @@
       </c>
       <c r="AK14" s="3">
         <f>+AK11*0.56</f>
-        <v>174138.09280000001</v>
+        <v>175732.78800000003</v>
       </c>
       <c r="AL14" s="3">
-        <f t="shared" ref="AL14:AR14" si="37">+AL11*0.56</f>
-        <v>194322.19844800004</v>
+        <f t="shared" ref="AL14:AR14" si="38">+AL11*0.56</f>
+        <v>195799.75212000002</v>
       </c>
       <c r="AM14" s="3">
-        <f t="shared" si="37"/>
-        <v>215994.21389728007</v>
+        <f t="shared" si="38"/>
+        <v>217351.48407560005</v>
       </c>
       <c r="AN14" s="3">
-        <f t="shared" si="37"/>
-        <v>241441.29442595688</v>
+        <f t="shared" si="38"/>
+        <v>242613.61068058806</v>
       </c>
       <c r="AO14" s="3">
-        <f t="shared" si="37"/>
-        <v>271555.57853201957</v>
+        <f t="shared" si="38"/>
+        <v>272456.87434901699</v>
       </c>
       <c r="AP14" s="3">
-        <f t="shared" si="37"/>
-        <v>301136.7681646854</v>
+        <f t="shared" si="38"/>
+        <v>301833.67981685244</v>
       </c>
       <c r="AQ14" s="3">
-        <f t="shared" si="37"/>
-        <v>334806.40589946706</v>
+        <f t="shared" si="38"/>
+        <v>335238.66818770883</v>
       </c>
       <c r="AR14" s="3">
-        <f t="shared" si="37"/>
-        <v>373221.67855405324</v>
+        <f t="shared" si="38"/>
+        <v>373315.63028966793</v>
       </c>
     </row>
     <row r="15" spans="1:44" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -2586,7 +2573,7 @@
         <v>31562</v>
       </c>
       <c r="AJ15" s="3">
-        <f t="shared" ref="AJ15:AJ17" si="38">SUM(O15:R15)</f>
+        <f t="shared" ref="AJ15:AJ17" si="39">SUM(O15:R15)</f>
         <v>39500</v>
       </c>
       <c r="AK15" s="3">
@@ -2594,31 +2581,31 @@
         <v>41475</v>
       </c>
       <c r="AL15" s="3">
-        <f t="shared" ref="AL15:AR15" si="39">+AK15*1.05</f>
+        <f t="shared" ref="AL15:AR15" si="40">+AK15*1.05</f>
         <v>43548.75</v>
       </c>
       <c r="AM15" s="3">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>45726.1875</v>
       </c>
       <c r="AN15" s="3">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>48012.496875000004</v>
       </c>
       <c r="AO15" s="3">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>50413.121718750008</v>
       </c>
       <c r="AP15" s="3">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>52933.77780468751</v>
       </c>
       <c r="AQ15" s="3">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>55580.466694921888</v>
       </c>
       <c r="AR15" s="3">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v>58359.490029667984</v>
       </c>
     </row>
@@ -2697,7 +2684,7 @@
         <v>22912</v>
       </c>
       <c r="AJ16" s="3">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>26567</v>
       </c>
       <c r="AK16" s="3">
@@ -2705,31 +2692,31 @@
         <v>27895.350000000002</v>
       </c>
       <c r="AL16" s="3">
-        <f t="shared" ref="AL16:AR16" si="40">+AK16*1.05</f>
+        <f t="shared" ref="AL16:AR16" si="41">+AK16*1.05</f>
         <v>29290.117500000004</v>
       </c>
       <c r="AM16" s="3">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>30754.623375000006</v>
       </c>
       <c r="AN16" s="3">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>32292.354543750007</v>
       </c>
       <c r="AO16" s="3">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>33906.972270937506</v>
       </c>
       <c r="AP16" s="3">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>35602.320884484383</v>
       </c>
       <c r="AQ16" s="3">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>37382.436928708601</v>
       </c>
       <c r="AR16" s="3">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v>39251.558775144033</v>
       </c>
     </row>
@@ -2808,7 +2795,7 @@
         <v>13510</v>
       </c>
       <c r="AJ17" s="3">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v>15724</v>
       </c>
       <c r="AK17" s="3">
@@ -2816,31 +2803,31 @@
         <v>16510.2</v>
       </c>
       <c r="AL17" s="3">
-        <f t="shared" ref="AL17:AR17" si="41">+AK17*1.05</f>
+        <f t="shared" ref="AL17:AR17" si="42">+AK17*1.05</f>
         <v>17335.710000000003</v>
       </c>
       <c r="AM17" s="3">
-        <f t="shared" si="41"/>
+        <f t="shared" si="42"/>
         <v>18202.495500000005</v>
       </c>
       <c r="AN17" s="3">
-        <f t="shared" si="41"/>
+        <f t="shared" si="42"/>
         <v>19112.620275000005</v>
       </c>
       <c r="AO17" s="3">
-        <f t="shared" si="41"/>
+        <f t="shared" si="42"/>
         <v>20068.251288750005</v>
       </c>
       <c r="AP17" s="3">
-        <f t="shared" si="41"/>
+        <f t="shared" si="42"/>
         <v>21071.663853187507</v>
       </c>
       <c r="AQ17" s="3">
-        <f t="shared" si="41"/>
+        <f t="shared" si="42"/>
         <v>22125.247045846882</v>
       </c>
       <c r="AR17" s="3">
-        <f t="shared" si="41"/>
+        <f t="shared" si="42"/>
         <v>23231.509398139227</v>
       </c>
     </row>
@@ -2849,26 +2836,26 @@
         <v>26</v>
       </c>
       <c r="C18" s="11">
-        <f t="shared" ref="C18" si="42">SUM(C15:C17)</f>
+        <f t="shared" ref="C18" si="43">SUM(C15:C17)</f>
         <v>12022</v>
       </c>
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
       <c r="F18" s="11"/>
       <c r="G18" s="11">
-        <f t="shared" ref="G18" si="43">SUM(G15:G17)</f>
+        <f t="shared" ref="G18" si="44">SUM(G15:G17)</f>
         <v>14200</v>
       </c>
       <c r="H18" s="11">
-        <f t="shared" ref="H18" si="44">SUM(H15:H17)</f>
+        <f t="shared" ref="H18" si="45">SUM(H15:H17)</f>
         <v>13361</v>
       </c>
       <c r="I18" s="11">
-        <f t="shared" ref="I18" si="45">SUM(I15:I17)</f>
+        <f t="shared" ref="I18" si="46">SUM(I15:I17)</f>
         <v>13843</v>
       </c>
       <c r="J18" s="11">
-        <f t="shared" ref="J18" si="46">SUM(J15:J17)</f>
+        <f t="shared" ref="J18" si="47">SUM(J15:J17)</f>
         <v>15167</v>
       </c>
       <c r="K18" s="11">
@@ -2876,27 +2863,27 @@
         <v>14774</v>
       </c>
       <c r="L18" s="11">
-        <f t="shared" ref="L18:O18" si="47">SUM(L15:L17)</f>
+        <f t="shared" ref="L18:O18" si="48">SUM(L15:L17)</f>
         <v>16292</v>
       </c>
       <c r="M18" s="11">
-        <f t="shared" si="47"/>
+        <f t="shared" si="48"/>
         <v>16466</v>
       </c>
       <c r="N18" s="11">
-        <f t="shared" si="47"/>
+        <f t="shared" si="48"/>
         <v>20452</v>
       </c>
       <c r="O18" s="11">
-        <f t="shared" si="47"/>
+        <f t="shared" si="48"/>
         <v>18318</v>
       </c>
       <c r="P18" s="11">
-        <f t="shared" ref="P18:Q18" si="48">SUM(P15:P17)</f>
+        <f t="shared" ref="P18:Q18" si="49">SUM(P15:P17)</f>
         <v>20128</v>
       </c>
       <c r="Q18" s="11">
-        <f t="shared" si="48"/>
+        <f t="shared" si="49"/>
         <v>20799</v>
       </c>
       <c r="R18" s="11">
@@ -2912,23 +2899,23 @@
         <v>23814</v>
       </c>
       <c r="AC18" s="3">
-        <f t="shared" ref="AC18:AG18" si="49">SUM(AC15:AC17)</f>
+        <f t="shared" ref="AC18:AG18" si="50">SUM(AC15:AC17)</f>
         <v>27465</v>
       </c>
       <c r="AD18" s="3">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v>31418</v>
       </c>
       <c r="AE18" s="3">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v>36390</v>
       </c>
       <c r="AF18" s="3">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v>45878</v>
       </c>
       <c r="AG18" s="3">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v>54033</v>
       </c>
       <c r="AH18" s="3">
@@ -2936,43 +2923,43 @@
         <v>56571</v>
       </c>
       <c r="AI18" s="3">
-        <f t="shared" ref="AI18:AK18" si="50">SUM(AI15:AI17)</f>
+        <f t="shared" ref="AI18:AK18" si="51">SUM(AI15:AI17)</f>
         <v>67984</v>
       </c>
       <c r="AJ18" s="3">
-        <f t="shared" si="50"/>
+        <f t="shared" si="51"/>
         <v>81791</v>
       </c>
       <c r="AK18" s="3">
-        <f t="shared" si="50"/>
+        <f t="shared" si="51"/>
         <v>85880.55</v>
       </c>
       <c r="AL18" s="3">
-        <f t="shared" ref="AL18:AR18" si="51">SUM(AL15:AL17)</f>
+        <f t="shared" ref="AL18:AR18" si="52">SUM(AL15:AL17)</f>
         <v>90174.577500000014</v>
       </c>
       <c r="AM18" s="3">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>94683.306375000015</v>
       </c>
       <c r="AN18" s="3">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>99417.47169375002</v>
       </c>
       <c r="AO18" s="3">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>104388.34527843751</v>
       </c>
       <c r="AP18" s="3">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>109607.7625423594</v>
       </c>
       <c r="AQ18" s="3">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>115088.15066947739</v>
       </c>
       <c r="AR18" s="3">
-        <f t="shared" si="51"/>
+        <f t="shared" si="52"/>
         <v>120842.55820295124</v>
       </c>
     </row>
@@ -2981,42 +2968,42 @@
         <v>27</v>
       </c>
       <c r="C19" s="11">
-        <f t="shared" ref="C19" si="52">C14-C18</f>
+        <f t="shared" ref="C19" si="53">C14-C18</f>
         <v>8305</v>
       </c>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
       <c r="F19" s="11"/>
       <c r="G19" s="11">
-        <f t="shared" ref="G19" si="53">G14-G18</f>
+        <f t="shared" ref="G19" si="54">G14-G18</f>
         <v>7977</v>
       </c>
       <c r="H19" s="11">
-        <f t="shared" ref="H19" si="54">H14-H18</f>
+        <f t="shared" ref="H19" si="55">H14-H18</f>
         <v>6383</v>
       </c>
       <c r="I19" s="11">
-        <f t="shared" ref="I19" si="55">I14-I18</f>
+        <f t="shared" ref="I19" si="56">I14-I18</f>
         <v>11213</v>
       </c>
       <c r="J19" s="11">
-        <f t="shared" ref="J19" si="56">J14-J18</f>
+        <f t="shared" ref="J19" si="57">J14-J18</f>
         <v>15651</v>
       </c>
       <c r="K19" s="11">
-        <f t="shared" ref="K19:N19" si="57">K14-K18</f>
+        <f t="shared" ref="K19:N19" si="58">K14-K18</f>
         <v>16437</v>
       </c>
       <c r="L19" s="11">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>19361</v>
       </c>
       <c r="M19" s="11">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>21031</v>
       </c>
       <c r="N19" s="11">
-        <f t="shared" si="57"/>
+        <f t="shared" si="58"/>
         <v>21885</v>
       </c>
       <c r="O19" s="11">
@@ -3024,15 +3011,15 @@
         <v>20094</v>
       </c>
       <c r="P19" s="11">
-        <f t="shared" ref="P19:R19" si="58">P14-P18</f>
+        <f t="shared" ref="P19:R19" si="59">P14-P18</f>
         <v>19453</v>
       </c>
       <c r="Q19" s="11">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>17135</v>
       </c>
       <c r="R19" s="11">
-        <f t="shared" si="58"/>
+        <f t="shared" si="59"/>
         <v>18160</v>
       </c>
       <c r="S19" s="11"/>
@@ -3044,23 +3031,23 @@
         <v>16496</v>
       </c>
       <c r="AC19" s="3">
-        <f t="shared" ref="AC19:AG19" si="59">AC14-AC18</f>
+        <f t="shared" ref="AC19:AG19" si="60">AC14-AC18</f>
         <v>19360</v>
       </c>
       <c r="AD19" s="3">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>23716</v>
       </c>
       <c r="AE19" s="3">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>28882</v>
       </c>
       <c r="AF19" s="3">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>31392</v>
       </c>
       <c r="AG19" s="3">
-        <f t="shared" si="59"/>
+        <f t="shared" si="60"/>
         <v>35928</v>
       </c>
       <c r="AH19" s="3">
@@ -3068,44 +3055,44 @@
         <v>41224</v>
       </c>
       <c r="AI19" s="3">
-        <f t="shared" ref="AI19:AK19" si="60">AI14-AI18</f>
+        <f t="shared" ref="AI19:AK19" si="61">AI14-AI18</f>
         <v>78714</v>
       </c>
       <c r="AJ19" s="3">
-        <f t="shared" si="60"/>
+        <f t="shared" si="61"/>
         <v>74842</v>
       </c>
       <c r="AK19" s="3">
-        <f t="shared" si="60"/>
-        <v>88257.54280000001</v>
+        <f t="shared" si="61"/>
+        <v>89852.238000000027</v>
       </c>
       <c r="AL19" s="3">
-        <f t="shared" ref="AL19:AR19" si="61">AL14-AL18</f>
-        <v>104147.62094800003</v>
+        <f t="shared" ref="AL19:AR19" si="62">AL14-AL18</f>
+        <v>105625.17462000001</v>
       </c>
       <c r="AM19" s="3">
-        <f t="shared" si="61"/>
-        <v>121310.90752228006</v>
+        <f t="shared" si="62"/>
+        <v>122668.17770060003</v>
       </c>
       <c r="AN19" s="3">
-        <f t="shared" si="61"/>
-        <v>142023.82273220684</v>
+        <f t="shared" si="62"/>
+        <v>143196.13898683805</v>
       </c>
       <c r="AO19" s="3">
-        <f t="shared" si="61"/>
-        <v>167167.23325358206</v>
+        <f t="shared" si="62"/>
+        <v>168068.52907057948</v>
       </c>
       <c r="AP19" s="3">
-        <f t="shared" si="61"/>
-        <v>191529.00562232599</v>
+        <f t="shared" si="62"/>
+        <v>192225.91727449303</v>
       </c>
       <c r="AQ19" s="3">
-        <f t="shared" si="61"/>
-        <v>219718.25522998968</v>
+        <f t="shared" si="62"/>
+        <v>220150.51751823144</v>
       </c>
       <c r="AR19" s="3">
-        <f t="shared" si="61"/>
-        <v>252379.120351102</v>
+        <f t="shared" si="62"/>
+        <v>252473.07208671668</v>
       </c>
     </row>
     <row r="20" spans="2:101" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -3183,7 +3170,7 @@
         <v>12020</v>
       </c>
       <c r="AJ20" s="3">
-        <f t="shared" ref="AJ20:AJ22" si="62">SUM(O20:R20)</f>
+        <f t="shared" ref="AJ20:AJ22" si="63">SUM(O20:R20)</f>
         <v>-3514</v>
       </c>
       <c r="AK20" s="3">
@@ -3191,32 +3178,32 @@
         <v>1295.53</v>
       </c>
       <c r="AL20" s="3">
-        <f t="shared" ref="AL20:AR20" si="63">+AK37*$AU$29</f>
-        <v>2029.86519696</v>
+        <f t="shared" ref="AL20:AR20" si="64">+AK37*$AU$29</f>
+        <v>2042.9416976000002</v>
       </c>
       <c r="AM20" s="3">
-        <f t="shared" si="63"/>
-        <v>2900.5205833486725</v>
+        <f t="shared" si="64"/>
+        <v>2925.8202514043205</v>
       </c>
       <c r="AN20" s="3">
-        <f t="shared" si="63"/>
-        <v>3919.0542938148278</v>
+        <f t="shared" si="64"/>
+        <v>3955.6910346107566</v>
       </c>
       <c r="AO20" s="3">
-        <f t="shared" si="63"/>
-        <v>5115.7858854282058</v>
+        <f t="shared" si="64"/>
+        <v>5162.3360407866367</v>
       </c>
       <c r="AP20" s="3">
-        <f t="shared" si="63"/>
-        <v>6528.5066423680892</v>
+        <f t="shared" si="64"/>
+        <v>6582.8291346998385</v>
       </c>
       <c r="AQ20" s="3">
-        <f t="shared" si="63"/>
-        <v>8152.5782429385808</v>
+        <f t="shared" si="64"/>
+        <v>8213.0608552552203</v>
       </c>
       <c r="AR20" s="3">
-        <f t="shared" si="63"/>
-        <v>10021.119077416592</v>
+        <f t="shared" si="64"/>
+        <v>10085.64219791781</v>
       </c>
     </row>
     <row r="21" spans="2:101" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -3224,26 +3211,26 @@
         <v>29</v>
       </c>
       <c r="C21" s="11">
-        <f t="shared" ref="C21" si="64">C19+C20</f>
+        <f t="shared" ref="C21" si="65">C19+C20</f>
         <v>9843</v>
       </c>
       <c r="D21" s="11"/>
       <c r="E21" s="11"/>
       <c r="F21" s="11"/>
       <c r="G21" s="11">
-        <f t="shared" ref="G21" si="65">G19+G20</f>
+        <f t="shared" ref="G21" si="66">G19+G20</f>
         <v>7757</v>
       </c>
       <c r="H21" s="11">
-        <f t="shared" ref="H21" si="66">H19+H20</f>
+        <f t="shared" ref="H21" si="67">H19+H20</f>
         <v>8277</v>
       </c>
       <c r="I21" s="11">
-        <f t="shared" ref="I21" si="67">I19+I20</f>
+        <f t="shared" ref="I21" si="68">I19+I20</f>
         <v>13359</v>
       </c>
       <c r="J21" s="11">
-        <f t="shared" ref="J21" si="68">J19+J20</f>
+        <f t="shared" ref="J21" si="69">J19+J20</f>
         <v>18689</v>
       </c>
       <c r="K21" s="11">
@@ -3251,31 +3238,31 @@
         <v>21283</v>
       </c>
       <c r="L21" s="11">
-        <f t="shared" ref="L21:O21" si="69">L19+L20</f>
+        <f t="shared" ref="L21:O21" si="70">L19+L20</f>
         <v>21625</v>
       </c>
       <c r="M21" s="11">
-        <f t="shared" si="69"/>
+        <f t="shared" si="70"/>
         <v>23064</v>
       </c>
       <c r="N21" s="11">
-        <f t="shared" si="69"/>
+        <f t="shared" si="70"/>
         <v>24402</v>
       </c>
       <c r="O21" s="11">
-        <f t="shared" si="69"/>
+        <f t="shared" si="70"/>
         <v>18934</v>
       </c>
       <c r="P21" s="11">
-        <f t="shared" ref="P21:R21" si="70">P19+P20</f>
+        <f t="shared" ref="P21:R21" si="71">P19+P20</f>
         <v>19014</v>
       </c>
       <c r="Q21" s="11">
-        <f t="shared" si="70"/>
+        <f t="shared" si="71"/>
         <v>16233</v>
       </c>
       <c r="R21" s="11">
-        <f t="shared" si="70"/>
+        <f t="shared" si="71"/>
         <v>17147</v>
       </c>
       <c r="S21" s="11"/>
@@ -3283,27 +3270,27 @@
       <c r="U21" s="11"/>
       <c r="V21" s="11"/>
       <c r="AB21" s="3">
-        <f>+AB19+AB20</f>
+        <f t="shared" ref="AB21:AG21" si="72">+AB19+AB20</f>
         <v>17259</v>
       </c>
       <c r="AC21" s="3">
-        <f>+AC19+AC20</f>
+        <f t="shared" si="72"/>
         <v>19651</v>
       </c>
       <c r="AD21" s="3">
-        <f>+AD19+AD20</f>
+        <f t="shared" si="72"/>
         <v>24150</v>
       </c>
       <c r="AE21" s="3">
-        <f>+AE19+AE20</f>
+        <f t="shared" si="72"/>
         <v>29929</v>
       </c>
       <c r="AF21" s="3">
-        <f>+AF19+AF20</f>
+        <f t="shared" si="72"/>
         <v>39984</v>
       </c>
       <c r="AG21" s="3">
-        <f>+AG19+AG20</f>
+        <f t="shared" si="72"/>
         <v>41322</v>
       </c>
       <c r="AH21" s="3">
@@ -3311,44 +3298,44 @@
         <v>48082</v>
       </c>
       <c r="AI21" s="3">
-        <f t="shared" ref="AI21:AK21" si="71">AI19+AI20</f>
+        <f t="shared" ref="AI21:AK21" si="73">AI19+AI20</f>
         <v>90734</v>
       </c>
       <c r="AJ21" s="3">
-        <f t="shared" si="71"/>
+        <f t="shared" si="73"/>
         <v>71328</v>
       </c>
       <c r="AK21" s="3">
-        <f t="shared" si="71"/>
-        <v>89553.072800000009</v>
+        <f t="shared" si="73"/>
+        <v>91147.768000000025</v>
       </c>
       <c r="AL21" s="3">
-        <f t="shared" ref="AL21:AR21" si="72">AL19+AL20</f>
-        <v>106177.48614496003</v>
+        <f t="shared" ref="AL21:AR21" si="74">AL19+AL20</f>
+        <v>107668.11631760001</v>
       </c>
       <c r="AM21" s="3">
-        <f t="shared" si="72"/>
-        <v>124211.42810562873</v>
+        <f t="shared" si="74"/>
+        <v>125593.99795200436</v>
       </c>
       <c r="AN21" s="3">
-        <f t="shared" si="72"/>
-        <v>145942.87702602166</v>
+        <f t="shared" si="74"/>
+        <v>147151.83002144881</v>
       </c>
       <c r="AO21" s="3">
-        <f t="shared" si="72"/>
-        <v>172283.01913901026</v>
+        <f t="shared" si="74"/>
+        <v>173230.86511136612</v>
       </c>
       <c r="AP21" s="3">
-        <f t="shared" si="72"/>
-        <v>198057.51226469409</v>
+        <f t="shared" si="74"/>
+        <v>198808.74640919286</v>
       </c>
       <c r="AQ21" s="3">
-        <f t="shared" si="72"/>
-        <v>227870.83347292827</v>
+        <f t="shared" si="74"/>
+        <v>228363.57837348667</v>
       </c>
       <c r="AR21" s="3">
-        <f t="shared" si="72"/>
-        <v>262400.23942851857</v>
+        <f t="shared" si="74"/>
+        <v>262558.71428463451</v>
       </c>
     </row>
     <row r="22" spans="2:101" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -3426,40 +3413,40 @@
         <v>14701</v>
       </c>
       <c r="AJ22" s="3">
-        <f t="shared" si="62"/>
+        <f t="shared" si="63"/>
         <v>11356</v>
       </c>
       <c r="AK22" s="3">
         <f>+AK21*0.18</f>
-        <v>16119.553104000001</v>
+        <v>16406.598240000003</v>
       </c>
       <c r="AL22" s="3">
-        <f t="shared" ref="AL22:AR22" si="73">+AL21*0.18</f>
-        <v>19111.947506092805</v>
+        <f t="shared" ref="AL22:AR22" si="75">+AL21*0.18</f>
+        <v>19380.260937168001</v>
       </c>
       <c r="AM22" s="3">
-        <f t="shared" si="73"/>
-        <v>22358.057059013172</v>
+        <f t="shared" si="75"/>
+        <v>22606.919631360783</v>
       </c>
       <c r="AN22" s="3">
-        <f t="shared" si="73"/>
-        <v>26269.717864683898</v>
+        <f t="shared" si="75"/>
+        <v>26487.329403860786</v>
       </c>
       <c r="AO22" s="3">
-        <f t="shared" si="73"/>
-        <v>31010.943445021843</v>
+        <f t="shared" si="75"/>
+        <v>31181.555720045901</v>
       </c>
       <c r="AP22" s="3">
-        <f t="shared" si="73"/>
-        <v>35650.352207644937</v>
+        <f t="shared" si="75"/>
+        <v>35785.574353654716</v>
       </c>
       <c r="AQ22" s="3">
-        <f t="shared" si="73"/>
-        <v>41016.750025127083</v>
+        <f t="shared" si="75"/>
+        <v>41105.444107227602</v>
       </c>
       <c r="AR22" s="3">
-        <f t="shared" si="73"/>
-        <v>47232.043097133341</v>
+        <f t="shared" si="75"/>
+        <v>47260.568571234209</v>
       </c>
     </row>
     <row r="23" spans="2:101" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -3467,26 +3454,26 @@
         <v>31</v>
       </c>
       <c r="C23" s="11">
-        <f t="shared" ref="C23" si="74">C21-C22</f>
+        <f t="shared" ref="C23" si="76">C21-C22</f>
         <v>8354</v>
       </c>
       <c r="D23" s="11"/>
       <c r="E23" s="11"/>
       <c r="F23" s="11"/>
       <c r="G23" s="11">
-        <f t="shared" ref="G23" si="75">G21-G22</f>
+        <f t="shared" ref="G23" si="77">G21-G22</f>
         <v>6836</v>
       </c>
       <c r="H23" s="11">
-        <f t="shared" ref="H23" si="76">H21-H22</f>
+        <f t="shared" ref="H23" si="78">H21-H22</f>
         <v>6959</v>
       </c>
       <c r="I23" s="11">
-        <f t="shared" ref="I23" si="77">I21-I22</f>
+        <f t="shared" ref="I23" si="79">I21-I22</f>
         <v>11247</v>
       </c>
       <c r="J23" s="11">
-        <f t="shared" ref="J23" si="78">J21-J22</f>
+        <f t="shared" ref="J23" si="80">J21-J22</f>
         <v>15227</v>
       </c>
       <c r="K23" s="11">
@@ -3494,31 +3481,31 @@
         <v>17930</v>
       </c>
       <c r="L23" s="11">
-        <f t="shared" ref="L23:O23" si="79">L21-L22</f>
+        <f t="shared" ref="L23:O23" si="81">L21-L22</f>
         <v>18165</v>
       </c>
       <c r="M23" s="11">
-        <f t="shared" si="79"/>
+        <f t="shared" si="81"/>
         <v>18936</v>
       </c>
       <c r="N23" s="11">
-        <f t="shared" si="79"/>
+        <f t="shared" si="81"/>
         <v>20642</v>
       </c>
       <c r="O23" s="11">
-        <f t="shared" si="79"/>
+        <f t="shared" si="81"/>
         <v>16436</v>
       </c>
       <c r="P23" s="11">
-        <f t="shared" ref="P23:R23" si="80">P21-P22</f>
+        <f t="shared" ref="P23:R23" si="82">P21-P22</f>
         <v>16002</v>
       </c>
       <c r="Q23" s="11">
-        <f t="shared" si="80"/>
+        <f t="shared" si="82"/>
         <v>13910</v>
       </c>
       <c r="R23" s="11">
-        <f t="shared" si="80"/>
+        <f t="shared" si="82"/>
         <v>13624</v>
       </c>
       <c r="S23" s="11"/>
@@ -3526,27 +3513,27 @@
       <c r="U23" s="11"/>
       <c r="V23" s="11"/>
       <c r="AB23" s="3">
-        <f>+AB21-AB22</f>
+        <f t="shared" ref="AB23:AG23" si="83">+AB21-AB22</f>
         <v>13620</v>
       </c>
       <c r="AC23" s="3">
-        <f>+AC21-AC22</f>
+        <f t="shared" si="83"/>
         <v>16348</v>
       </c>
       <c r="AD23" s="3">
-        <f>+AD21-AD22</f>
+        <f t="shared" si="83"/>
         <v>19478</v>
       </c>
       <c r="AE23" s="3">
-        <f>+AE21-AE22</f>
+        <f t="shared" si="83"/>
         <v>15398</v>
       </c>
       <c r="AF23" s="3">
-        <f>+AF21-AF22</f>
+        <f t="shared" si="83"/>
         <v>35807</v>
       </c>
       <c r="AG23" s="3">
-        <f>+AG21-AG22</f>
+        <f t="shared" si="83"/>
         <v>36040</v>
       </c>
       <c r="AH23" s="3">
@@ -3554,272 +3541,272 @@
         <v>40269</v>
       </c>
       <c r="AI23" s="3">
-        <f t="shared" ref="AI23:AK23" si="81">AI21-AI22</f>
+        <f t="shared" ref="AI23:AK23" si="84">AI21-AI22</f>
         <v>76033</v>
       </c>
       <c r="AJ23" s="3">
-        <f t="shared" si="81"/>
+        <f t="shared" si="84"/>
         <v>59972</v>
       </c>
       <c r="AK23" s="3">
-        <f t="shared" si="81"/>
-        <v>73433.519696000003</v>
+        <f t="shared" si="84"/>
+        <v>74741.169760000019</v>
       </c>
       <c r="AL23" s="3">
-        <f t="shared" ref="AL23:AR23" si="82">AL21-AL22</f>
-        <v>87065.53863886722</v>
+        <f t="shared" ref="AL23:AR23" si="85">AL21-AL22</f>
+        <v>88287.855380432011</v>
       </c>
       <c r="AM23" s="3">
-        <f t="shared" si="82"/>
-        <v>101853.37104661556</v>
+        <f t="shared" si="85"/>
+        <v>102987.07832064357</v>
       </c>
       <c r="AN23" s="3">
-        <f t="shared" si="82"/>
-        <v>119673.15916133775</v>
+        <f t="shared" si="85"/>
+        <v>120664.50061758803</v>
       </c>
       <c r="AO23" s="3">
-        <f t="shared" si="82"/>
-        <v>141272.07569398842</v>
+        <f t="shared" si="85"/>
+        <v>142049.30939132022</v>
       </c>
       <c r="AP23" s="3">
-        <f t="shared" si="82"/>
-        <v>162407.16005704916</v>
+        <f t="shared" si="85"/>
+        <v>163023.17205553813</v>
       </c>
       <c r="AQ23" s="3">
-        <f t="shared" si="82"/>
-        <v>186854.08344780118</v>
+        <f t="shared" si="85"/>
+        <v>187258.13426625906</v>
       </c>
       <c r="AR23" s="3">
-        <f t="shared" si="82"/>
-        <v>215168.19633138523</v>
+        <f t="shared" si="85"/>
+        <v>215298.1457134003</v>
       </c>
       <c r="AS23" s="3">
         <f>+AR23*(1+$AU$27)</f>
-        <v>213016.51436807137</v>
+        <v>213145.16425626629</v>
       </c>
       <c r="AT23" s="3">
-        <f t="shared" ref="AT23:CW23" si="83">+AS23*(1+$AU$27)</f>
-        <v>210886.34922439064</v>
+        <f t="shared" ref="AT23:CW23" si="86">+AS23*(1+$AU$27)</f>
+        <v>211013.71261370362</v>
       </c>
       <c r="AU23" s="3">
-        <f t="shared" si="83"/>
-        <v>208777.48573214674</v>
+        <f t="shared" si="86"/>
+        <v>208903.57548756659</v>
       </c>
       <c r="AV23" s="3">
-        <f t="shared" si="83"/>
-        <v>206689.71087482528</v>
+        <f t="shared" si="86"/>
+        <v>206814.53973269093</v>
       </c>
       <c r="AW23" s="3">
-        <f t="shared" si="83"/>
-        <v>204622.81376607702</v>
+        <f t="shared" si="86"/>
+        <v>204746.39433536402</v>
       </c>
       <c r="AX23" s="3">
-        <f t="shared" si="83"/>
-        <v>202576.58562841624</v>
+        <f t="shared" si="86"/>
+        <v>202698.93039201037</v>
       </c>
       <c r="AY23" s="3">
-        <f t="shared" si="83"/>
-        <v>200550.81977213209</v>
+        <f t="shared" si="86"/>
+        <v>200671.94108809027</v>
       </c>
       <c r="AZ23" s="3">
-        <f t="shared" si="83"/>
-        <v>198545.31157441076</v>
+        <f t="shared" si="86"/>
+        <v>198665.22167720937</v>
       </c>
       <c r="BA23" s="3">
-        <f t="shared" si="83"/>
-        <v>196559.85845866665</v>
+        <f t="shared" si="86"/>
+        <v>196678.56946043728</v>
       </c>
       <c r="BB23" s="3">
-        <f t="shared" si="83"/>
-        <v>194594.25987407999</v>
+        <f t="shared" si="86"/>
+        <v>194711.78376583292</v>
       </c>
       <c r="BC23" s="3">
-        <f t="shared" si="83"/>
-        <v>192648.31727533918</v>
+        <f t="shared" si="86"/>
+        <v>192764.6659281746</v>
       </c>
       <c r="BD23" s="3">
-        <f t="shared" si="83"/>
-        <v>190721.8341025858</v>
+        <f t="shared" si="86"/>
+        <v>190837.01926889285</v>
       </c>
       <c r="BE23" s="3">
-        <f t="shared" si="83"/>
-        <v>188814.61576155992</v>
+        <f t="shared" si="86"/>
+        <v>188928.64907620393</v>
       </c>
       <c r="BF23" s="3">
-        <f t="shared" si="83"/>
-        <v>186926.46960394431</v>
+        <f t="shared" si="86"/>
+        <v>187039.36258544188</v>
       </c>
       <c r="BG23" s="3">
-        <f t="shared" si="83"/>
-        <v>185057.20490790487</v>
+        <f t="shared" si="86"/>
+        <v>185168.96895958745</v>
       </c>
       <c r="BH23" s="3">
-        <f t="shared" si="83"/>
-        <v>183206.63285882582</v>
+        <f t="shared" si="86"/>
+        <v>183317.27926999159</v>
       </c>
       <c r="BI23" s="3">
-        <f t="shared" si="83"/>
-        <v>181374.56653023756</v>
+        <f t="shared" si="86"/>
+        <v>181484.10647729167</v>
       </c>
       <c r="BJ23" s="3">
-        <f t="shared" si="83"/>
-        <v>179560.82086493517</v>
+        <f t="shared" si="86"/>
+        <v>179669.26541251875</v>
       </c>
       <c r="BK23" s="3">
-        <f t="shared" si="83"/>
-        <v>177765.21265628582</v>
+        <f t="shared" si="86"/>
+        <v>177872.57275839357</v>
       </c>
       <c r="BL23" s="3">
-        <f t="shared" si="83"/>
-        <v>175987.56052972295</v>
+        <f t="shared" si="86"/>
+        <v>176093.84703080961</v>
       </c>
       <c r="BM23" s="3">
-        <f t="shared" si="83"/>
-        <v>174227.68492442573</v>
+        <f t="shared" si="86"/>
+        <v>174332.90856050153</v>
       </c>
       <c r="BN23" s="3">
-        <f t="shared" si="83"/>
-        <v>172485.40807518148</v>
+        <f t="shared" si="86"/>
+        <v>172589.57947489651</v>
       </c>
       <c r="BO23" s="3">
-        <f t="shared" si="83"/>
-        <v>170760.55399442965</v>
+        <f t="shared" si="86"/>
+        <v>170863.68368014754</v>
       </c>
       <c r="BP23" s="3">
-        <f t="shared" si="83"/>
-        <v>169052.94845448536</v>
+        <f t="shared" si="86"/>
+        <v>169155.04684334606</v>
       </c>
       <c r="BQ23" s="3">
-        <f t="shared" si="83"/>
-        <v>167362.41896994051</v>
+        <f t="shared" si="86"/>
+        <v>167463.49637491259</v>
       </c>
       <c r="BR23" s="3">
-        <f t="shared" si="83"/>
-        <v>165688.79478024109</v>
+        <f t="shared" si="86"/>
+        <v>165788.86141116347</v>
       </c>
       <c r="BS23" s="3">
-        <f t="shared" si="83"/>
-        <v>164031.90683243869</v>
+        <f t="shared" si="86"/>
+        <v>164130.97279705183</v>
       </c>
       <c r="BT23" s="3">
-        <f t="shared" si="83"/>
-        <v>162391.58776411432</v>
+        <f t="shared" si="86"/>
+        <v>162489.66306908132</v>
       </c>
       <c r="BU23" s="3">
-        <f t="shared" si="83"/>
-        <v>160767.67188647317</v>
+        <f t="shared" si="86"/>
+        <v>160864.76643839051</v>
       </c>
       <c r="BV23" s="3">
-        <f t="shared" si="83"/>
-        <v>159159.99516760843</v>
+        <f t="shared" si="86"/>
+        <v>159256.11877400661</v>
       </c>
       <c r="BW23" s="3">
-        <f t="shared" si="83"/>
-        <v>157568.39521593234</v>
+        <f t="shared" si="86"/>
+        <v>157663.55758626654</v>
       </c>
       <c r="BX23" s="3">
-        <f t="shared" si="83"/>
-        <v>155992.711263773</v>
+        <f t="shared" si="86"/>
+        <v>156086.92201040388</v>
       </c>
       <c r="BY23" s="3">
-        <f t="shared" si="83"/>
-        <v>154432.78415113527</v>
+        <f t="shared" si="86"/>
+        <v>154526.05279029984</v>
       </c>
       <c r="BZ23" s="3">
-        <f t="shared" si="83"/>
-        <v>152888.45630962393</v>
+        <f t="shared" si="86"/>
+        <v>152980.79226239683</v>
       </c>
       <c r="CA23" s="3">
-        <f t="shared" si="83"/>
-        <v>151359.57174652768</v>
+        <f t="shared" si="86"/>
+        <v>151450.98433977287</v>
       </c>
       <c r="CB23" s="3">
-        <f t="shared" si="83"/>
-        <v>149845.97602906241</v>
+        <f t="shared" si="86"/>
+        <v>149936.47449637513</v>
       </c>
       <c r="CC23" s="3">
-        <f t="shared" si="83"/>
-        <v>148347.51626877178</v>
+        <f t="shared" si="86"/>
+        <v>148437.10975141136</v>
       </c>
       <c r="CD23" s="3">
-        <f t="shared" si="83"/>
-        <v>146864.04110608407</v>
+        <f t="shared" si="86"/>
+        <v>146952.73865389725</v>
       </c>
       <c r="CE23" s="3">
-        <f t="shared" si="83"/>
-        <v>145395.40069502321</v>
+        <f t="shared" si="86"/>
+        <v>145483.21126735827</v>
       </c>
       <c r="CF23" s="3">
-        <f t="shared" si="83"/>
-        <v>143941.44668807299</v>
+        <f t="shared" si="86"/>
+        <v>144028.37915468469</v>
       </c>
       <c r="CG23" s="3">
-        <f t="shared" si="83"/>
-        <v>142502.03222119226</v>
+        <f t="shared" si="86"/>
+        <v>142588.09536313784</v>
       </c>
       <c r="CH23" s="3">
-        <f t="shared" si="83"/>
-        <v>141077.01189898033</v>
+        <f t="shared" si="86"/>
+        <v>141162.21440950644</v>
       </c>
       <c r="CI23" s="3">
-        <f t="shared" si="83"/>
-        <v>139666.24177999052</v>
+        <f t="shared" si="86"/>
+        <v>139750.59226541137</v>
       </c>
       <c r="CJ23" s="3">
-        <f t="shared" si="83"/>
-        <v>138269.57936219062</v>
+        <f t="shared" si="86"/>
+        <v>138353.08634275725</v>
       </c>
       <c r="CK23" s="3">
-        <f t="shared" si="83"/>
-        <v>136886.88356856871</v>
+        <f t="shared" si="86"/>
+        <v>136969.55547932966</v>
       </c>
       <c r="CL23" s="3">
-        <f t="shared" si="83"/>
-        <v>135518.01473288302</v>
+        <f t="shared" si="86"/>
+        <v>135599.85992453637</v>
       </c>
       <c r="CM23" s="3">
-        <f t="shared" si="83"/>
-        <v>134162.8345855542</v>
+        <f t="shared" si="86"/>
+        <v>134243.86132529101</v>
       </c>
       <c r="CN23" s="3">
-        <f t="shared" si="83"/>
-        <v>132821.20623969866</v>
+        <f t="shared" si="86"/>
+        <v>132901.4227120381</v>
       </c>
       <c r="CO23" s="3">
-        <f t="shared" si="83"/>
-        <v>131492.99417730168</v>
+        <f t="shared" si="86"/>
+        <v>131572.40848491772</v>
       </c>
       <c r="CP23" s="3">
-        <f t="shared" si="83"/>
-        <v>130178.06423552865</v>
+        <f t="shared" si="86"/>
+        <v>130256.68440006854</v>
       </c>
       <c r="CQ23" s="3">
-        <f t="shared" si="83"/>
-        <v>128876.28359317337</v>
+        <f t="shared" si="86"/>
+        <v>128954.11755606785</v>
       </c>
       <c r="CR23" s="3">
-        <f t="shared" si="83"/>
-        <v>127587.52075724164</v>
+        <f t="shared" si="86"/>
+        <v>127664.57638050718</v>
       </c>
       <c r="CS23" s="3">
-        <f t="shared" si="83"/>
-        <v>126311.64554966922</v>
+        <f t="shared" si="86"/>
+        <v>126387.9306167021</v>
       </c>
       <c r="CT23" s="3">
-        <f t="shared" si="83"/>
-        <v>125048.52909417253</v>
+        <f t="shared" si="86"/>
+        <v>125124.05131053508</v>
       </c>
       <c r="CU23" s="3">
-        <f t="shared" si="83"/>
-        <v>123798.0438032308</v>
+        <f t="shared" si="86"/>
+        <v>123872.81079742973</v>
       </c>
       <c r="CV23" s="3">
-        <f t="shared" si="83"/>
-        <v>122560.0633651985</v>
+        <f t="shared" si="86"/>
+        <v>122634.08268945543</v>
       </c>
       <c r="CW23" s="3">
-        <f t="shared" si="83"/>
-        <v>121334.4627315465</v>
+        <f t="shared" si="86"/>
+        <v>121407.74186256088</v>
       </c>
     </row>
     <row r="24" spans="2:101" s="7" customFormat="1" x14ac:dyDescent="0.2">
@@ -3827,42 +3814,42 @@
         <v>32</v>
       </c>
       <c r="C24" s="14">
-        <f t="shared" ref="C24" si="84">C23/C25</f>
+        <f t="shared" ref="C24" si="87">C23/C25</f>
         <v>11.919318455824756</v>
       </c>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
       <c r="F24" s="14"/>
       <c r="G24" s="14">
-        <f t="shared" ref="G24" si="85">G23/G25</f>
+        <f t="shared" ref="G24" si="88">G23/G25</f>
         <v>9.8748026411774639</v>
       </c>
       <c r="H24" s="14">
-        <f t="shared" ref="H24" si="86">H23/H25</f>
+        <f t="shared" ref="H24" si="89">H23/H25</f>
         <v>10.129194904399265</v>
       </c>
       <c r="I24" s="14">
-        <f t="shared" ref="I24" si="87">I23/I25</f>
+        <f t="shared" ref="I24" si="90">I23/I25</f>
         <v>16.398605528022852</v>
       </c>
       <c r="J24" s="14">
-        <f t="shared" ref="J24" si="88">J23/J25</f>
+        <f t="shared" ref="J24" si="91">J23/J25</f>
         <v>22.295301836540162</v>
       </c>
       <c r="K24" s="14">
-        <f t="shared" ref="K24:N24" si="89">K23/K25</f>
+        <f t="shared" ref="K24:N24" si="92">K23/K25</f>
         <v>26.287585896482916</v>
       </c>
       <c r="L24" s="14">
-        <f t="shared" si="89"/>
+        <f t="shared" si="92"/>
         <v>1.3364479105356091</v>
       </c>
       <c r="M24" s="14">
-        <f t="shared" si="89"/>
+        <f t="shared" si="92"/>
         <v>27.990344690984287</v>
       </c>
       <c r="N24" s="14">
-        <f t="shared" si="89"/>
+        <f t="shared" si="92"/>
         <v>30.69474329100823</v>
       </c>
       <c r="O24" s="14">
@@ -3870,15 +3857,15 @@
         <v>24.621339792764896</v>
       </c>
       <c r="P24" s="14">
-        <f t="shared" ref="P24:R24" si="90">P23/P25</f>
+        <f t="shared" ref="P24:R24" si="93">P23/P25</f>
         <v>1.2087015635622025</v>
       </c>
       <c r="Q24" s="14">
-        <f t="shared" si="90"/>
+        <f t="shared" si="93"/>
         <v>1.0620752844162786</v>
       </c>
       <c r="R24" s="14">
-        <f t="shared" si="90"/>
+        <f t="shared" si="93"/>
         <v>1.0522901058160192</v>
       </c>
       <c r="S24" s="14"/>
@@ -3899,35 +3886,35 @@
       </c>
       <c r="AK24" s="17">
         <f>AK23/AK25</f>
-        <v>5.6080380594150139</v>
+        <v>5.7079018730748681</v>
       </c>
       <c r="AL24" s="17">
-        <f t="shared" ref="AL24:AR24" si="91">AL23/AL25</f>
-        <v>6.6491005248224839</v>
+        <f t="shared" ref="AL24:AR24" si="94">AL23/AL25</f>
+        <v>6.7424475254256553</v>
       </c>
       <c r="AM24" s="17">
-        <f t="shared" si="91"/>
-        <v>7.778431207897734</v>
+        <f t="shared" si="94"/>
+        <v>7.8650111998047683</v>
       </c>
       <c r="AN24" s="17">
-        <f t="shared" si="91"/>
-        <v>9.1393090518548288</v>
+        <f t="shared" si="94"/>
+        <v>9.2150167210438116</v>
       </c>
       <c r="AO24" s="17">
-        <f t="shared" si="91"/>
-        <v>10.788794824274246</v>
+        <f t="shared" si="94"/>
+        <v>10.848151316700879</v>
       </c>
       <c r="AP24" s="17">
-        <f t="shared" si="91"/>
-        <v>12.402858238198393</v>
+        <f t="shared" si="94"/>
+        <v>12.449902404770878</v>
       </c>
       <c r="AQ24" s="17">
-        <f t="shared" si="91"/>
-        <v>14.269843197907582</v>
+        <f t="shared" si="94"/>
+        <v>14.3007001196135</v>
       </c>
       <c r="AR24" s="17">
-        <f t="shared" si="91"/>
-        <v>16.432161214626063</v>
+        <f t="shared" si="94"/>
+        <v>16.44208530764455</v>
       </c>
     </row>
     <row r="25" spans="2:101" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -4001,31 +3988,31 @@
         <v>13094.333333333334</v>
       </c>
       <c r="AL25" s="3">
-        <f t="shared" ref="AL25:AR25" si="92">+AK25</f>
+        <f t="shared" ref="AL25:AR25" si="95">+AK25</f>
         <v>13094.333333333334</v>
       </c>
       <c r="AM25" s="3">
-        <f t="shared" si="92"/>
+        <f t="shared" si="95"/>
         <v>13094.333333333334</v>
       </c>
       <c r="AN25" s="3">
-        <f t="shared" si="92"/>
+        <f t="shared" si="95"/>
         <v>13094.333333333334</v>
       </c>
       <c r="AO25" s="3">
-        <f t="shared" si="92"/>
+        <f t="shared" si="95"/>
         <v>13094.333333333334</v>
       </c>
       <c r="AP25" s="3">
-        <f t="shared" si="92"/>
+        <f t="shared" si="95"/>
         <v>13094.333333333334</v>
       </c>
       <c r="AQ25" s="3">
-        <f t="shared" si="92"/>
+        <f t="shared" si="95"/>
         <v>13094.333333333334</v>
       </c>
       <c r="AR25" s="3">
-        <f t="shared" si="92"/>
+        <f t="shared" si="95"/>
         <v>13094.333333333334</v>
       </c>
     </row>
@@ -4042,19 +4029,19 @@
       <c r="I27" s="16"/>
       <c r="J27" s="16"/>
       <c r="K27" s="16">
-        <f t="shared" ref="K27:L27" si="93">K11/G11-1</f>
+        <f t="shared" ref="K27:L27" si="96">K11/G11-1</f>
         <v>0.34391020189994892</v>
       </c>
       <c r="L27" s="16">
-        <f t="shared" si="93"/>
+        <f t="shared" si="96"/>
         <v>0.61579235971486024</v>
       </c>
       <c r="M27" s="16">
-        <f t="shared" ref="M27" si="94">M11/I11-1</f>
+        <f t="shared" ref="M27" si="97">M11/I11-1</f>
         <v>0.41030472353973102</v>
       </c>
       <c r="N27" s="16">
-        <f t="shared" ref="N27" si="95">N11/J11-1</f>
+        <f t="shared" ref="N27" si="98">N11/J11-1</f>
         <v>0.32386024113325607</v>
       </c>
       <c r="O27" s="16">
@@ -4062,11 +4049,11 @@
         <v>0.22954405756228069</v>
       </c>
       <c r="P27" s="16">
-        <f t="shared" ref="P27:U27" si="96">P11/L11-1</f>
+        <f t="shared" ref="P27:U27" si="99">P11/L11-1</f>
         <v>0.12613122171945701</v>
       </c>
       <c r="Q27" s="16">
-        <f t="shared" si="96"/>
+        <f t="shared" si="99"/>
         <v>6.1027672840074931E-2</v>
       </c>
       <c r="R27" s="16">
@@ -4074,92 +4061,92 @@
         <v>9.5984069034185104E-3</v>
       </c>
       <c r="S27" s="16">
-        <f t="shared" si="96"/>
+        <f t="shared" si="99"/>
         <v>0.10948331887488805</v>
       </c>
       <c r="T27" s="16">
-        <f t="shared" si="96"/>
+        <f t="shared" si="99"/>
         <v>0.11002640453469192</v>
       </c>
       <c r="U27" s="16">
-        <f t="shared" si="96"/>
+        <f t="shared" si="99"/>
         <v>0.10828185607595664</v>
       </c>
       <c r="V27" s="16">
         <f>V11/R11-1</f>
-        <v>0.10659793814432983</v>
+        <v>0.13494108983799702</v>
       </c>
       <c r="AA27" s="18">
-        <f>AA11/Z11-1</f>
+        <f t="shared" ref="AA27:AJ27" si="100">AA11/Z11-1</f>
         <v>0.2059123786355046</v>
       </c>
       <c r="AB27" s="18">
-        <f>AB11/AA11-1</f>
+        <f t="shared" si="100"/>
         <v>0.18880023055170292</v>
       </c>
       <c r="AC27" s="18">
-        <f>AC11/AB11-1</f>
+        <f t="shared" si="100"/>
         <v>0.13617975485219924</v>
       </c>
       <c r="AD27" s="18">
-        <f>AD11/AC11-1</f>
+        <f t="shared" si="100"/>
         <v>0.20380322447292265</v>
       </c>
       <c r="AE27" s="18">
-        <f>AE11/AD11-1</f>
+        <f t="shared" si="100"/>
         <v>0.22801090038993266</v>
       </c>
       <c r="AF27" s="18">
-        <f>AF11/AE11-1</f>
+        <f t="shared" si="100"/>
         <v>0.23421586757475987</v>
       </c>
       <c r="AG27" s="18">
-        <f>AG11/AF11-1</f>
+        <f t="shared" si="100"/>
         <v>0.18300089899794614</v>
       </c>
       <c r="AH27" s="18">
-        <f>AH11/AG11-1</f>
+        <f t="shared" si="100"/>
         <v>0.12770532012826141</v>
       </c>
       <c r="AI27" s="18">
-        <f>AI11/AH11-1</f>
+        <f t="shared" si="100"/>
         <v>0.41150076427049154</v>
       </c>
       <c r="AJ27" s="18">
-        <f>AJ11/AI11-1</f>
+        <f t="shared" si="100"/>
         <v>9.7808156437157789E-2</v>
       </c>
       <c r="AK27" s="18">
-        <f t="shared" ref="AK27:AR27" si="97">AK11/AJ11-1</f>
-        <v>9.9438826740584574E-2</v>
+        <f t="shared" ref="AK27:AR27" si="101">AK11/AJ11-1</f>
+        <v>0.10950709952057047</v>
       </c>
       <c r="AL27" s="18">
-        <f t="shared" si="97"/>
-        <v>0.11590861782999839</v>
+        <f t="shared" si="101"/>
+        <v>0.11419021087857528</v>
       </c>
       <c r="AM27" s="18">
-        <f t="shared" si="97"/>
-        <v>0.11152619526934493</v>
+        <f t="shared" si="101"/>
+        <v>0.11007027190918817</v>
       </c>
       <c r="AN27" s="18">
-        <f t="shared" si="97"/>
-        <v>0.11781371393947904</v>
+        <f t="shared" si="101"/>
+        <v>0.11622707207373484</v>
       </c>
       <c r="AO27" s="18">
-        <f t="shared" si="97"/>
-        <v>0.12472714817761998</v>
+        <f t="shared" si="101"/>
+        <v>0.12300737615136903</v>
       </c>
       <c r="AP27" s="18">
-        <f t="shared" si="97"/>
-        <v>0.10893235849757321</v>
+        <f t="shared" si="101"/>
+        <v>0.10782185451560244</v>
       </c>
       <c r="AQ27" s="18">
-        <f t="shared" si="97"/>
-        <v>0.11180845813012263</v>
+        <f t="shared" si="101"/>
+        <v>0.11067349538701565</v>
       </c>
       <c r="AR27" s="18">
-        <f t="shared" si="97"/>
-        <v>0.11473876239429304</v>
+        <f t="shared" si="101"/>
+        <v>0.11358165305870616</v>
       </c>
       <c r="AT27" s="18" t="s">
         <v>72</v>
@@ -4216,19 +4203,19 @@
       <c r="I29" s="15"/>
       <c r="J29" s="15"/>
       <c r="K29" s="15">
-        <f t="shared" ref="K29" si="98">+K9/G9-1</f>
+        <f t="shared" ref="K29" si="102">+K9/G9-1</f>
         <v>0.30107746306423966</v>
       </c>
       <c r="L29" s="15">
-        <f t="shared" ref="L29:N29" si="99">+L9/H9-1</f>
+        <f t="shared" ref="L29:N29" si="103">+L9/H9-1</f>
         <v>0.68136404146535945</v>
       </c>
       <c r="M29" s="15">
-        <f t="shared" si="99"/>
+        <f t="shared" si="103"/>
         <v>0.43997266307236682</v>
       </c>
       <c r="N29" s="15">
-        <f t="shared" si="99"/>
+        <f t="shared" si="103"/>
         <v>0.35727047613077145</v>
       </c>
       <c r="O29" s="15">
@@ -4252,55 +4239,55 @@
       <c r="U29" s="15"/>
       <c r="V29" s="15"/>
       <c r="AF29" s="5">
-        <f t="shared" ref="AF29:AJ29" si="100">+AF9/AE9-1</f>
+        <f t="shared" ref="AF29:AJ29" si="104">+AF9/AE9-1</f>
         <v>0.22181318130380601</v>
       </c>
       <c r="AG29" s="5">
-        <f t="shared" si="100"/>
+        <f t="shared" si="104"/>
         <v>0.15028840742824978</v>
       </c>
       <c r="AH29" s="5">
-        <f t="shared" si="100"/>
+        <f t="shared" si="104"/>
         <v>6.0612546501554343E-2</v>
       </c>
       <c r="AI29" s="5">
-        <f t="shared" si="100"/>
+        <f t="shared" si="104"/>
         <v>0.43136783840402826</v>
       </c>
       <c r="AJ29" s="5">
-        <f t="shared" si="100"/>
+        <f t="shared" si="104"/>
         <v>9.0627118985438182E-2</v>
       </c>
       <c r="AK29" s="5">
         <f>+AK9/AJ9-1</f>
+        <v>0.10711357340720218</v>
+      </c>
+      <c r="AL29" s="15">
+        <f t="shared" ref="AL29:AR29" si="105">+AL9/AK9-1</f>
         <v>0.10000000000000009</v>
       </c>
-      <c r="AL29" s="15">
-        <f t="shared" ref="AL29:AR29" si="101">+AL9/AK9-1</f>
+      <c r="AM29" s="15">
+        <f t="shared" si="105"/>
         <v>0.10000000000000009</v>
       </c>
-      <c r="AM29" s="15">
-        <f t="shared" si="101"/>
+      <c r="AN29" s="15">
+        <f t="shared" si="105"/>
         <v>0.10000000000000009</v>
       </c>
-      <c r="AN29" s="15">
-        <f t="shared" si="101"/>
+      <c r="AO29" s="15">
+        <f t="shared" si="105"/>
         <v>0.10000000000000009</v>
       </c>
-      <c r="AO29" s="15">
-        <f t="shared" si="101"/>
+      <c r="AP29" s="15">
+        <f t="shared" si="105"/>
         <v>0.10000000000000009</v>
       </c>
-      <c r="AP29" s="15">
-        <f t="shared" si="101"/>
+      <c r="AQ29" s="15">
+        <f t="shared" si="105"/>
         <v>0.10000000000000009</v>
       </c>
-      <c r="AQ29" s="15">
-        <f t="shared" si="101"/>
-        <v>0.10000000000000009</v>
-      </c>
       <c r="AR29" s="15">
-        <f t="shared" si="101"/>
+        <f t="shared" si="105"/>
         <v>0.10000000000000009</v>
       </c>
       <c r="AT29" s="5" t="s">
@@ -4323,31 +4310,31 @@
       <c r="I30" s="15"/>
       <c r="J30" s="15"/>
       <c r="K30" s="15">
-        <f t="shared" ref="K30" si="102">+K8/G8-1</f>
+        <f t="shared" ref="K30" si="106">+K8/G8-1</f>
         <v>0.48712233779098568</v>
       </c>
       <c r="L30" s="15">
-        <f t="shared" ref="L30:Q30" si="103">+L8/H8-1</f>
+        <f t="shared" ref="L30:Q30" si="107">+L8/H8-1</f>
         <v>0.83683105981112282</v>
       </c>
       <c r="M30" s="15">
-        <f t="shared" si="103"/>
+        <f t="shared" si="107"/>
         <v>0.4304149295215407</v>
       </c>
       <c r="N30" s="15">
-        <f t="shared" si="103"/>
+        <f t="shared" si="107"/>
         <v>0.25388525780682647</v>
       </c>
       <c r="O30" s="15">
-        <f t="shared" si="103"/>
+        <f t="shared" si="107"/>
         <v>0.143880099916736</v>
       </c>
       <c r="P30" s="15">
-        <f t="shared" si="103"/>
+        <f t="shared" si="107"/>
         <v>4.8271922307911996E-2</v>
       </c>
       <c r="Q30" s="15">
-        <f t="shared" si="103"/>
+        <f t="shared" si="107"/>
         <v>-1.8598195697432374E-2</v>
       </c>
       <c r="R30" s="15">
@@ -4359,19 +4346,19 @@
       <c r="U30" s="15"/>
       <c r="V30" s="15"/>
       <c r="AF30" s="5">
-        <f t="shared" ref="AF30:AI30" si="104">+AF8/AE8-1</f>
+        <f t="shared" ref="AF30:AI30" si="108">+AF8/AE8-1</f>
         <v>0.36871165644171788</v>
       </c>
       <c r="AG30" s="5">
-        <f t="shared" si="104"/>
+        <f t="shared" si="108"/>
         <v>0.35804571940833707</v>
       </c>
       <c r="AH30" s="5">
-        <f t="shared" si="104"/>
+        <f t="shared" si="108"/>
         <v>0.30516865799722748</v>
       </c>
       <c r="AI30" s="5">
-        <f t="shared" si="104"/>
+        <f t="shared" si="108"/>
         <v>0.45888124620675708</v>
       </c>
       <c r="AJ30" s="5">
@@ -4380,34 +4367,34 @@
       </c>
       <c r="AK30" s="5">
         <f>+AK8/AJ8-1</f>
+        <v>8.5962452552747814E-2</v>
+      </c>
+      <c r="AL30" s="15">
+        <f t="shared" ref="AL30:AR30" si="109">+AL8/AK8-1</f>
         <v>5.0000000000000044E-2</v>
       </c>
-      <c r="AL30" s="15">
-        <f t="shared" ref="AL30:AR30" si="105">+AL8/AK8-1</f>
+      <c r="AM30" s="15">
+        <f t="shared" si="109"/>
         <v>5.0000000000000044E-2</v>
       </c>
-      <c r="AM30" s="15">
-        <f t="shared" si="105"/>
+      <c r="AN30" s="15">
+        <f t="shared" si="109"/>
         <v>5.0000000000000044E-2</v>
       </c>
-      <c r="AN30" s="15">
-        <f t="shared" si="105"/>
+      <c r="AO30" s="15">
+        <f t="shared" si="109"/>
         <v>5.0000000000000044E-2</v>
       </c>
-      <c r="AO30" s="15">
-        <f t="shared" si="105"/>
+      <c r="AP30" s="15">
+        <f t="shared" si="109"/>
         <v>5.0000000000000044E-2</v>
       </c>
-      <c r="AP30" s="15">
-        <f t="shared" si="105"/>
+      <c r="AQ30" s="15">
+        <f t="shared" si="109"/>
         <v>5.0000000000000044E-2</v>
       </c>
-      <c r="AQ30" s="15">
-        <f t="shared" si="105"/>
-        <v>5.0000000000000044E-2</v>
-      </c>
       <c r="AR30" s="15">
-        <f t="shared" si="105"/>
+        <f t="shared" si="109"/>
         <v>5.0000000000000044E-2</v>
       </c>
       <c r="AT30" s="5" t="s">
@@ -4415,7 +4402,7 @@
       </c>
       <c r="AU30" s="3">
         <f>NPV(AU28,AK23:CW23)+Main!L5-Main!L6</f>
-        <v>2137013.8680530442</v>
+        <v>2142891.2311289348</v>
       </c>
     </row>
     <row r="31" spans="2:101" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -4431,19 +4418,19 @@
       <c r="I31" s="15"/>
       <c r="J31" s="15"/>
       <c r="K31" s="15">
-        <f t="shared" ref="K31" si="106">K10/G10-1</f>
+        <f t="shared" ref="K31" si="110">K10/G10-1</f>
         <v>0.33980836693020566</v>
       </c>
       <c r="L31" s="15">
-        <f t="shared" ref="L31" si="107">L10/H10-1</f>
+        <f t="shared" ref="L31" si="111">L10/H10-1</f>
         <v>0.63090508988025484</v>
       </c>
       <c r="M31" s="15">
-        <f t="shared" ref="M31" si="108">M10/I10-1</f>
+        <f t="shared" ref="M31" si="112">M10/I10-1</f>
         <v>0.40661921875367013</v>
       </c>
       <c r="N31" s="15">
-        <f t="shared" ref="N31" si="109">N10/J10-1</f>
+        <f t="shared" ref="N31" si="113">N10/J10-1</f>
         <v>0.31257919921320898</v>
       </c>
       <c r="O31" s="15">
@@ -4451,11 +4438,11 @@
         <v>0.20114111532299028</v>
       </c>
       <c r="P31" s="15">
-        <f t="shared" ref="P31:Q31" si="110">P10/L10-1</f>
+        <f t="shared" ref="P31:Q31" si="114">P10/L10-1</f>
         <v>0.10117931554138115</v>
       </c>
       <c r="Q31" s="15">
-        <f t="shared" si="110"/>
+        <f t="shared" si="114"/>
         <v>2.4931534299645897E-2</v>
       </c>
       <c r="R31" s="15">
@@ -4467,63 +4454,63 @@
       <c r="U31" s="15"/>
       <c r="V31" s="15"/>
       <c r="AF31" s="5">
-        <f t="shared" ref="AF31:AJ31" si="111">+AF10/AE10-1</f>
+        <f t="shared" ref="AF31:AJ31" si="115">+AF10/AE10-1</f>
         <v>0.22568104346846218</v>
       </c>
       <c r="AG31" s="5">
-        <f t="shared" si="111"/>
+        <f t="shared" si="115"/>
         <v>0.16319604057491333</v>
       </c>
       <c r="AH31" s="5">
-        <f t="shared" si="111"/>
+        <f t="shared" si="115"/>
         <v>0.11071957846204517</v>
       </c>
       <c r="AI31" s="5">
-        <f t="shared" si="111"/>
+        <f t="shared" si="115"/>
         <v>0.40853915260770313</v>
       </c>
       <c r="AJ31" s="5">
-        <f t="shared" si="111"/>
+        <f t="shared" si="115"/>
         <v>6.7355986005919188E-2</v>
       </c>
       <c r="AK31" s="5">
         <f>+AK10/AJ10-1</f>
-        <v>7.7159919219967898E-2</v>
+        <v>9.087181691963031E-2</v>
       </c>
       <c r="AL31" s="15">
-        <f t="shared" ref="AL31:AR31" si="112">+AL10/AK10-1</f>
-        <v>7.8052815516631568E-2</v>
+        <f t="shared" ref="AL31:AR31" si="116">+AL10/AK10-1</f>
+        <v>7.7817344505327846E-2</v>
       </c>
       <c r="AM31" s="15">
-        <f t="shared" si="112"/>
-        <v>7.8926787613141869E-2</v>
+        <f t="shared" si="116"/>
+        <v>7.8694942661178713E-2</v>
       </c>
       <c r="AN31" s="15">
-        <f t="shared" si="112"/>
-        <v>7.9780908994353084E-2</v>
+        <f t="shared" si="116"/>
+        <v>7.9553004436609065E-2</v>
       </c>
       <c r="AO31" s="15">
-        <f t="shared" si="112"/>
-        <v>8.0614365686686451E-2</v>
+        <f t="shared" si="116"/>
+        <v>8.0390688276103184E-2</v>
       </c>
       <c r="AP31" s="15">
-        <f t="shared" si="112"/>
-        <v>8.1426456360157662E-2</v>
+        <f t="shared" si="116"/>
+        <v>8.1207264673085033E-2</v>
       </c>
       <c r="AQ31" s="15">
-        <f t="shared" si="112"/>
-        <v>8.2216591293572172E-2</v>
+        <f t="shared" si="116"/>
+        <v>8.2002115452358915E-2</v>
       </c>
       <c r="AR31" s="15">
-        <f t="shared" si="112"/>
-        <v>8.2984290295815111E-2</v>
+        <f t="shared" si="116"/>
+        <v>8.2774731990183259E-2</v>
       </c>
       <c r="AT31" s="5" t="s">
         <v>76</v>
       </c>
       <c r="AU31" s="1">
         <f>+AU30/Main!L3</f>
-        <v>166.86295526298463</v>
+        <v>167.32187328249665</v>
       </c>
     </row>
     <row r="32" spans="2:101" s="5" customFormat="1" x14ac:dyDescent="0.2">
@@ -4539,19 +4526,19 @@
       <c r="I32" s="15"/>
       <c r="J32" s="15"/>
       <c r="K32" s="15">
-        <f t="shared" ref="K32" si="113">K5/G5-1</f>
+        <f t="shared" ref="K32" si="117">K5/G5-1</f>
         <v>0.4573280518545193</v>
       </c>
       <c r="L32" s="15">
-        <f t="shared" ref="L32" si="114">L5/H5-1</f>
+        <f t="shared" ref="L32" si="118">L5/H5-1</f>
         <v>0.53907549052211512</v>
       </c>
       <c r="M32" s="15">
-        <f t="shared" ref="M32" si="115">M5/I5-1</f>
+        <f t="shared" ref="M32" si="119">M5/I5-1</f>
         <v>0.44889663182346107</v>
       </c>
       <c r="N32" s="15">
-        <f t="shared" ref="N32" si="116">N5/J5-1</f>
+        <f t="shared" ref="N32" si="120">N5/J5-1</f>
         <v>0.44635865309318712</v>
       </c>
       <c r="O32" s="15">
@@ -4559,11 +4546,11 @@
         <v>0.4383493946132937</v>
       </c>
       <c r="P32" s="15">
-        <f t="shared" ref="P32:Q32" si="117">P5/L5-1</f>
+        <f t="shared" ref="P32:Q32" si="121">P5/L5-1</f>
         <v>0.35609334485738975</v>
       </c>
       <c r="Q32" s="15">
-        <f t="shared" si="117"/>
+        <f t="shared" si="121"/>
         <v>0.37635270541082155</v>
       </c>
       <c r="R32" s="15">
@@ -4575,55 +4562,55 @@
       <c r="U32" s="15"/>
       <c r="V32" s="15"/>
       <c r="AF32" s="5">
-        <f t="shared" ref="AF32:AJ32" si="118">+AF5/AE5-1</f>
+        <f t="shared" ref="AF32:AJ32" si="122">+AF5/AE5-1</f>
         <v>0.43934911242603558</v>
       </c>
       <c r="AG32" s="5">
-        <f t="shared" si="118"/>
+        <f t="shared" si="122"/>
         <v>0.52757793764988015</v>
       </c>
       <c r="AH32" s="5">
-        <f t="shared" si="118"/>
+        <f t="shared" si="122"/>
         <v>0.46434178066831122</v>
       </c>
       <c r="AI32" s="5">
-        <f t="shared" si="118"/>
+        <f t="shared" si="122"/>
         <v>0.47070985527222597</v>
       </c>
       <c r="AJ32" s="5">
-        <f t="shared" si="118"/>
+        <f t="shared" si="122"/>
         <v>0.36832239925023424</v>
       </c>
       <c r="AK32" s="5">
         <f>+AK5/AJ5-1</f>
+        <v>0.36008371385083704</v>
+      </c>
+      <c r="AL32" s="15">
+        <f t="shared" ref="AL32:AR32" si="123">+AL5/AK5-1</f>
         <v>0.39999999999999991</v>
       </c>
-      <c r="AL32" s="15">
-        <f t="shared" ref="AL32:AR32" si="119">+AL5/AK5-1</f>
-        <v>0.39999999999999991</v>
-      </c>
       <c r="AM32" s="15">
-        <f t="shared" si="119"/>
-        <v>0.30000000000000027</v>
+        <f t="shared" si="123"/>
+        <v>0.30000000000000004</v>
       </c>
       <c r="AN32" s="15">
-        <f t="shared" si="119"/>
+        <f t="shared" si="123"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="AO32" s="15">
-        <f t="shared" si="119"/>
+        <f t="shared" si="123"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="AP32" s="15">
-        <f t="shared" si="119"/>
+        <f t="shared" si="123"/>
         <v>0.19999999999999996</v>
       </c>
       <c r="AQ32" s="15">
-        <f t="shared" si="119"/>
+        <f t="shared" si="123"/>
         <v>0.19999999999999996</v>
       </c>
       <c r="AR32" s="15">
-        <f t="shared" si="119"/>
+        <f t="shared" si="123"/>
         <v>0.19999999999999996</v>
       </c>
     </row>
@@ -4636,19 +4623,19 @@
       <c r="E33" s="15"/>
       <c r="F33" s="15"/>
       <c r="G33" s="15">
-        <f t="shared" ref="G33:H33" si="120">G14/G11</f>
+        <f t="shared" ref="G33:H33" si="124">G14/G11</f>
         <v>0.53881289632887097</v>
       </c>
       <c r="H33" s="15">
-        <f t="shared" si="120"/>
+        <f t="shared" si="124"/>
         <v>0.51554952085019712</v>
       </c>
       <c r="I33" s="15">
-        <f t="shared" ref="I33" si="121">I14/I11</f>
+        <f t="shared" ref="I33" si="125">I14/I11</f>
         <v>0.54265479825872265</v>
       </c>
       <c r="J33" s="15">
-        <f t="shared" ref="J33" si="122">J14/J11</f>
+        <f t="shared" ref="J33" si="126">J14/J11</f>
         <v>0.54163590987380927</v>
       </c>
       <c r="K33" s="15">
@@ -4656,30 +4643,30 @@
         <v>0.56425136493473627</v>
       </c>
       <c r="L33" s="15">
-        <f t="shared" ref="L33:O33" si="123">L14/L11</f>
+        <f t="shared" ref="L33:O33" si="127">L14/L11</f>
         <v>0.57616354234001288</v>
       </c>
       <c r="M33" s="15">
-        <f t="shared" si="123"/>
+        <f t="shared" si="127"/>
         <v>0.57583156730857832</v>
       </c>
       <c r="N33" s="15">
-        <f t="shared" si="123"/>
+        <f t="shared" si="127"/>
         <v>0.56205774975107869</v>
       </c>
       <c r="O33" s="15">
-        <f t="shared" si="123"/>
+        <f t="shared" si="127"/>
         <v>0.5647909896928438</v>
       </c>
       <c r="P33" s="15">
-        <f t="shared" ref="P33:Q33" si="124">P14/P11</f>
+        <f t="shared" ref="P33:Q33" si="128">P14/P11</f>
         <v>0.56799885197675248</v>
       </c>
       <c r="Q33" s="15">
-        <f t="shared" si="124"/>
+        <f t="shared" si="128"/>
         <v>0.54903606785156023</v>
       </c>
-      <c r="R33" s="19">
+      <c r="R33" s="15">
         <f>R14/R11</f>
         <v>0.53526719966337055</v>
       </c>
@@ -4688,31 +4675,31 @@
       <c r="U33" s="15"/>
       <c r="V33" s="15"/>
       <c r="AB33" s="5">
-        <f t="shared" ref="AB33" si="125">AB14/AB11</f>
+        <f t="shared" ref="AB33" si="129">AB14/AB11</f>
         <v>0.6107483219951213</v>
       </c>
       <c r="AC33" s="5">
-        <f t="shared" ref="AC33" si="126">AC14/AC11</f>
+        <f t="shared" ref="AC33" si="130">AC14/AC11</f>
         <v>0.62442491565429592</v>
       </c>
       <c r="AD33" s="5">
-        <f t="shared" ref="AD33:AE33" si="127">AD14/AD11</f>
+        <f t="shared" ref="AD33:AE33" si="131">AD14/AD11</f>
         <v>0.61075416518964909</v>
       </c>
       <c r="AE33" s="5">
-        <f t="shared" si="127"/>
+        <f t="shared" si="131"/>
         <v>0.58880519597672631</v>
       </c>
       <c r="AF33" s="5">
-        <f t="shared" ref="AF33:AH33" si="128">AF14/AF11</f>
+        <f t="shared" ref="AF33:AH33" si="132">AF14/AF11</f>
         <v>0.5647607422945643</v>
       </c>
       <c r="AG33" s="5">
-        <f t="shared" si="128"/>
+        <f t="shared" si="132"/>
         <v>0.5558054331910266</v>
       </c>
       <c r="AH33" s="5">
-        <f t="shared" si="128"/>
+        <f t="shared" si="132"/>
         <v>0.53578374706207854</v>
       </c>
       <c r="AI33" s="5">
@@ -4724,35 +4711,35 @@
         <v>0.55379442503783116</v>
       </c>
       <c r="AK33" s="5">
-        <f t="shared" ref="AJ33:AK33" si="129">AK14/AK11</f>
+        <f t="shared" ref="AK33" si="133">AK14/AK11</f>
         <v>0.56000000000000005</v>
       </c>
       <c r="AL33" s="15">
-        <f t="shared" ref="AL33:AR33" si="130">AL14/AL11</f>
+        <f t="shared" ref="AL33:AR33" si="134">AL14/AL11</f>
         <v>0.56000000000000005</v>
       </c>
       <c r="AM33" s="15">
-        <f t="shared" si="130"/>
+        <f t="shared" si="134"/>
         <v>0.56000000000000005</v>
       </c>
       <c r="AN33" s="15">
-        <f t="shared" si="130"/>
+        <f t="shared" si="134"/>
         <v>0.56000000000000005</v>
       </c>
       <c r="AO33" s="15">
-        <f t="shared" si="130"/>
+        <f t="shared" si="134"/>
         <v>0.56000000000000005</v>
       </c>
       <c r="AP33" s="15">
-        <f t="shared" si="130"/>
+        <f t="shared" si="134"/>
         <v>0.56000000000000005</v>
       </c>
       <c r="AQ33" s="15">
-        <f t="shared" si="130"/>
+        <f t="shared" si="134"/>
         <v>0.56000000000000005</v>
       </c>
       <c r="AR33" s="15">
-        <f t="shared" si="130"/>
+        <f t="shared" si="134"/>
         <v>0.56000000000000005</v>
       </c>
     </row>
@@ -4765,7 +4752,7 @@
       <c r="E34" s="15"/>
       <c r="F34" s="15"/>
       <c r="G34" s="15">
-        <f t="shared" ref="G34" si="131">+G22/G21</f>
+        <f t="shared" ref="G34" si="135">+G22/G21</f>
         <v>0.11873146835116669</v>
       </c>
       <c r="H34" s="15">
@@ -4773,39 +4760,39 @@
         <v>0.15923643832306392</v>
       </c>
       <c r="I34" s="15">
-        <f t="shared" ref="I34:Q34" si="132">+I22/I21</f>
+        <f t="shared" ref="I34:Q34" si="136">+I22/I21</f>
         <v>0.15809566584325174</v>
       </c>
       <c r="J34" s="15">
-        <f t="shared" si="132"/>
+        <f t="shared" si="136"/>
         <v>0.18524265610787094</v>
       </c>
       <c r="K34" s="15">
-        <f t="shared" si="132"/>
+        <f t="shared" si="136"/>
         <v>0.15754357938260583</v>
       </c>
       <c r="L34" s="15">
-        <f t="shared" si="132"/>
+        <f t="shared" si="136"/>
         <v>0.16</v>
       </c>
       <c r="M34" s="15">
-        <f t="shared" si="132"/>
+        <f t="shared" si="136"/>
         <v>0.17898022892819979</v>
       </c>
       <c r="N34" s="15">
-        <f t="shared" si="132"/>
+        <f t="shared" si="136"/>
         <v>0.15408573067781328</v>
       </c>
       <c r="O34" s="15">
-        <f t="shared" si="132"/>
+        <f t="shared" si="136"/>
         <v>0.13193197422625963</v>
       </c>
       <c r="P34" s="15">
-        <f t="shared" si="132"/>
+        <f t="shared" si="136"/>
         <v>0.15840959293152415</v>
       </c>
       <c r="Q34" s="15">
-        <f t="shared" si="132"/>
+        <f t="shared" si="136"/>
         <v>0.14310355448777182</v>
       </c>
       <c r="R34" s="15">
@@ -4817,35 +4804,35 @@
       <c r="U34" s="15"/>
       <c r="V34" s="15"/>
       <c r="AB34" s="15">
-        <f t="shared" ref="AB34" si="133">+AB22/AB21</f>
+        <f t="shared" ref="AB34" si="137">+AB22/AB21</f>
         <v>0.21084651486181122</v>
       </c>
       <c r="AC34" s="15">
-        <f t="shared" ref="AC34" si="134">+AC22/AC21</f>
+        <f t="shared" ref="AC34" si="138">+AC22/AC21</f>
         <v>0.16808304920869166</v>
       </c>
       <c r="AD34" s="15">
-        <f t="shared" ref="AD34:AE34" si="135">+AD22/AD21</f>
+        <f t="shared" ref="AD34:AE34" si="139">+AD22/AD21</f>
         <v>0.19345755693581781</v>
       </c>
       <c r="AE34" s="15">
-        <f t="shared" si="135"/>
+        <f t="shared" si="139"/>
         <v>0.48551572053860803</v>
       </c>
       <c r="AF34" s="15">
-        <f t="shared" ref="AF34:AH34" si="136">+AF22/AF21</f>
+        <f t="shared" ref="AF34:AH34" si="140">+AF22/AF21</f>
         <v>0.10446678671468587</v>
       </c>
       <c r="AG34" s="15">
-        <f t="shared" si="136"/>
+        <f t="shared" si="140"/>
         <v>0.12782537147282319</v>
       </c>
       <c r="AH34" s="15">
-        <f t="shared" si="136"/>
+        <f t="shared" si="140"/>
         <v>0.16249324071378063</v>
       </c>
       <c r="AI34" s="15">
-        <f t="shared" ref="AI34:AK34" si="137">+AI22/AI21</f>
+        <f t="shared" ref="AI34:AK34" si="141">+AI22/AI21</f>
         <v>0.16202305640663919</v>
       </c>
       <c r="AJ34" s="15">
@@ -4853,35 +4840,35 @@
         <v>0.1592081650964558</v>
       </c>
       <c r="AK34" s="15">
-        <f t="shared" si="137"/>
+        <f t="shared" si="141"/>
         <v>0.18</v>
       </c>
       <c r="AL34" s="15">
-        <f t="shared" ref="AL34:AR34" si="138">+AL22/AL21</f>
+        <f t="shared" ref="AL34:AR34" si="142">+AL22/AL21</f>
         <v>0.18</v>
       </c>
       <c r="AM34" s="15">
-        <f t="shared" si="138"/>
+        <f t="shared" si="142"/>
         <v>0.18</v>
       </c>
       <c r="AN34" s="15">
-        <f t="shared" si="138"/>
+        <f t="shared" si="142"/>
         <v>0.18</v>
       </c>
       <c r="AO34" s="15">
-        <f t="shared" si="138"/>
+        <f t="shared" si="142"/>
         <v>0.18</v>
       </c>
       <c r="AP34" s="15">
-        <f t="shared" si="138"/>
+        <f t="shared" si="142"/>
         <v>0.18000000000000002</v>
       </c>
       <c r="AQ34" s="15">
-        <f t="shared" si="138"/>
+        <f t="shared" si="142"/>
         <v>0.18</v>
       </c>
       <c r="AR34" s="15">
-        <f t="shared" si="138"/>
+        <f t="shared" si="142"/>
         <v>0.18</v>
       </c>
     </row>
@@ -4894,15 +4881,15 @@
       <c r="E35" s="15"/>
       <c r="F35" s="15"/>
       <c r="G35" s="15">
-        <f t="shared" ref="G35:H35" si="139">G9/G11</f>
+        <f t="shared" ref="G35:H35" si="143">G9/G11</f>
         <v>0.5953011492018756</v>
       </c>
       <c r="H35" s="15">
-        <f t="shared" si="139"/>
+        <f t="shared" si="143"/>
         <v>0.55667545760764547</v>
       </c>
       <c r="I35" s="15">
-        <f t="shared" ref="I35" si="140">I9/I11</f>
+        <f t="shared" ref="I35" si="144">I9/I11</f>
         <v>0.57041994239057459</v>
       </c>
       <c r="J35" s="15">
@@ -4910,31 +4897,31 @@
         <v>0.56070512144539353</v>
       </c>
       <c r="K35" s="15">
-        <f t="shared" ref="K35:O35" si="141">K9/K11</f>
+        <f t="shared" ref="K35:O35" si="145">K9/K11</f>
         <v>0.57632787359438842</v>
       </c>
       <c r="L35" s="15">
-        <f t="shared" si="141"/>
+        <f t="shared" si="145"/>
         <v>0.57926632191338079</v>
       </c>
       <c r="M35" s="15">
-        <f t="shared" si="141"/>
+        <f t="shared" si="145"/>
         <v>0.58241960748180222</v>
       </c>
       <c r="N35" s="15">
-        <f t="shared" si="141"/>
+        <f t="shared" si="145"/>
         <v>0.5748556256223033</v>
       </c>
       <c r="O35" s="15">
-        <f t="shared" si="141"/>
+        <f t="shared" si="145"/>
         <v>0.58252341532987306</v>
       </c>
       <c r="P35" s="15">
-        <f t="shared" ref="P35:Q35" si="142">P9/P11</f>
+        <f t="shared" ref="P35:Q35" si="146">P9/P11</f>
         <v>0.58389897395422252</v>
       </c>
       <c r="Q35" s="15">
-        <f t="shared" si="142"/>
+        <f t="shared" si="146"/>
         <v>0.57226596422161757</v>
       </c>
       <c r="R35" s="15">
@@ -4946,48 +4933,48 @@
       <c r="U35" s="15"/>
       <c r="V35" s="15"/>
       <c r="AH35" s="15">
-        <f t="shared" ref="AH35:AK35" si="143">AH9/AH11</f>
+        <f t="shared" ref="AH35:AK35" si="147">AH9/AH11</f>
         <v>0.57011839344316184</v>
       </c>
       <c r="AI35" s="15">
-        <f t="shared" si="143"/>
+        <f t="shared" si="147"/>
         <v>0.57814289096674776</v>
       </c>
       <c r="AJ35" s="15">
-        <f t="shared" si="143"/>
+        <f t="shared" si="147"/>
         <v>0.57436111386103605</v>
       </c>
       <c r="AK35" s="15">
-        <f t="shared" si="143"/>
-        <v>0.57465427805581204</v>
+        <f t="shared" si="147"/>
+        <v>0.57312205164582031</v>
       </c>
       <c r="AL35" s="15">
-        <f t="shared" ref="AL35:AR35" si="144">AL9/AL11</f>
-        <v>0.56646189101990851</v>
+        <f t="shared" ref="AL35:AR35" si="148">AL9/AL11</f>
+        <v>0.56582282868316036</v>
       </c>
       <c r="AM35" s="15">
-        <f t="shared" si="144"/>
-        <v>0.56058785008742684</v>
+        <f t="shared" si="148"/>
+        <v>0.56068982955557767</v>
       </c>
       <c r="AN35" s="15">
-        <f t="shared" si="144"/>
-        <v>0.55165420445857594</v>
+        <f t="shared" si="148"/>
+        <v>0.55253884083398586</v>
       </c>
       <c r="AO35" s="15">
-        <f t="shared" si="144"/>
-        <v>0.53952607606889824</v>
+        <f t="shared" si="148"/>
+        <v>0.54121881817048789</v>
       </c>
       <c r="AP35" s="15">
-        <f t="shared" si="144"/>
-        <v>0.53518023811646842</v>
+        <f t="shared" si="148"/>
+        <v>0.53739750444610135</v>
       </c>
       <c r="AQ35" s="15">
-        <f t="shared" si="144"/>
-        <v>0.52949611745013003</v>
+        <f t="shared" si="148"/>
+        <v>0.53223315163807794</v>
       </c>
       <c r="AR35" s="15">
-        <f t="shared" si="144"/>
-        <v>0.52249526870684604</v>
+        <f t="shared" si="148"/>
+        <v>0.52574183958023724</v>
       </c>
     </row>
     <row r="37" spans="2:44" x14ac:dyDescent="0.2">
@@ -4999,11 +4986,11 @@
         <v>124580</v>
       </c>
       <c r="N37" s="11">
-        <f t="shared" ref="N37:O37" si="145">+N38-N56</f>
+        <f t="shared" ref="N37:O37" si="149">+N38-N56</f>
         <v>154381</v>
       </c>
       <c r="O37" s="11">
-        <f t="shared" si="145"/>
+        <f t="shared" si="149"/>
         <v>149723</v>
       </c>
       <c r="P37" s="11">
@@ -5031,35 +5018,35 @@
       </c>
       <c r="AK37" s="3">
         <f>+AJ37+AK23</f>
-        <v>202986.519696</v>
+        <v>204294.16976000002</v>
       </c>
       <c r="AL37" s="3">
-        <f t="shared" ref="AL37:AR37" si="146">+AK37+AL23</f>
-        <v>290052.05833486724</v>
+        <f t="shared" ref="AL37:AR37" si="150">+AK37+AL23</f>
+        <v>292582.02514043206</v>
       </c>
       <c r="AM37" s="3">
-        <f t="shared" si="146"/>
-        <v>391905.42938148277</v>
+        <f t="shared" si="150"/>
+        <v>395569.10346107563</v>
       </c>
       <c r="AN37" s="3">
-        <f t="shared" si="146"/>
-        <v>511578.58854282054</v>
+        <f t="shared" si="150"/>
+        <v>516233.60407866363</v>
       </c>
       <c r="AO37" s="3">
-        <f t="shared" si="146"/>
-        <v>652850.66423680889</v>
+        <f t="shared" si="150"/>
+        <v>658282.91346998385</v>
       </c>
       <c r="AP37" s="3">
-        <f t="shared" si="146"/>
-        <v>815257.82429385802</v>
+        <f t="shared" si="150"/>
+        <v>821306.08552552201</v>
       </c>
       <c r="AQ37" s="3">
-        <f t="shared" si="146"/>
-        <v>1002111.9077416592</v>
+        <f t="shared" si="150"/>
+        <v>1008564.219791781</v>
       </c>
       <c r="AR37" s="3">
-        <f t="shared" si="146"/>
-        <v>1217280.1040730444</v>
+        <f t="shared" si="150"/>
+        <v>1223862.3655051813</v>
       </c>
     </row>
     <row r="38" spans="2:44" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -5769,47 +5756,47 @@
         <v>6836</v>
       </c>
       <c r="H62" s="11">
-        <f t="shared" ref="H62:R62" si="147">+H23</f>
+        <f t="shared" ref="H62:R62" si="151">+H23</f>
         <v>6959</v>
       </c>
       <c r="I62" s="11">
-        <f t="shared" si="147"/>
+        <f t="shared" si="151"/>
         <v>11247</v>
       </c>
       <c r="J62" s="11">
-        <f t="shared" si="147"/>
+        <f t="shared" si="151"/>
         <v>15227</v>
       </c>
       <c r="K62" s="11">
-        <f t="shared" si="147"/>
+        <f t="shared" si="151"/>
         <v>17930</v>
       </c>
       <c r="L62" s="11">
-        <f t="shared" si="147"/>
+        <f t="shared" si="151"/>
         <v>18165</v>
       </c>
       <c r="M62" s="11">
-        <f t="shared" si="147"/>
+        <f t="shared" si="151"/>
         <v>18936</v>
       </c>
       <c r="N62" s="11">
-        <f t="shared" si="147"/>
+        <f t="shared" si="151"/>
         <v>20642</v>
       </c>
       <c r="O62" s="11">
-        <f t="shared" si="147"/>
+        <f t="shared" si="151"/>
         <v>16436</v>
       </c>
       <c r="P62" s="11">
-        <f t="shared" si="147"/>
+        <f t="shared" si="151"/>
         <v>16002</v>
       </c>
       <c r="Q62" s="11">
-        <f t="shared" si="147"/>
+        <f t="shared" si="151"/>
         <v>13910</v>
       </c>
       <c r="R62" s="11">
-        <f t="shared" si="147"/>
+        <f t="shared" si="151"/>
         <v>13624</v>
       </c>
       <c r="S62" s="11"/>
@@ -6782,35 +6769,35 @@
         <v>334.49548143813797</v>
       </c>
       <c r="K92" s="11">
-        <f>+K11/K90*1000</f>
+        <f t="shared" ref="K92:R92" si="152">+K11/K90*1000</f>
         <v>395.11411121825779</v>
       </c>
       <c r="L92" s="11">
-        <f>+L11/L90*1000</f>
+        <f t="shared" si="152"/>
         <v>429.55517298828232</v>
       </c>
       <c r="M92" s="11">
-        <f>+M11/M90*1000</f>
+        <f t="shared" si="152"/>
         <v>434.03897939051376</v>
       </c>
       <c r="N92" s="11">
-        <f>+N11/N90*1000</f>
+        <f t="shared" si="152"/>
         <v>481.30990415335464</v>
       </c>
       <c r="O92" s="11">
-        <f>+O11/O90*1000</f>
+        <f t="shared" si="152"/>
         <v>414.93905043134475</v>
       </c>
       <c r="P92" s="11">
-        <f>+P11/P90*1000</f>
+        <f t="shared" si="152"/>
         <v>400.45628512648409</v>
       </c>
       <c r="Q92" s="11">
-        <f>+Q11/Q90*1000</f>
+        <f t="shared" si="152"/>
         <v>369.91310586307884</v>
       </c>
       <c r="R92" s="11">
-        <f>+R11/R90*1000</f>
+        <f t="shared" si="152"/>
         <v>399.76029521536634</v>
       </c>
     </row>

</xml_diff>